<commit_message>
Rewrite the publishing calendar from the live wave-2 patrol mix. [skip render]
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/ORION_Publishing_Calendar.xlsx
+++ b/ORION_Publishing_Calendar.xlsx
@@ -888,17 +888,17 @@
       <c r="F6" s="5" t="inlineStr"/>
       <c r="G6" s="5" t="inlineStr">
         <is>
-          <t>0828_patrol_theflood_916.mov</t>
+          <t>0827_theflood_916.mov</t>
         </is>
       </c>
       <c r="H6" s="7" t="inlineStr">
         <is>
-          <t>Not linked yet</t>
+          <t>Linked</t>
         </is>
       </c>
       <c r="I6" s="5" t="inlineStr">
         <is>
-          <t>Draft</t>
+          <t>Approved</t>
         </is>
       </c>
       <c r="J6" s="6" t="inlineStr">
@@ -1019,18 +1019,18 @@
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>GREAT WALL</t>
+          <t>GOLD DASH</t>
         </is>
       </c>
       <c r="E8" s="6" t="inlineStr">
         <is>
-          <t>nothing but walls today.</t>
-        </is>
-      </c>
-      <c r="F8" s="5" t="inlineStr"/>
+          <t>Commit the line. The landing is yours.</t>
+        </is>
+      </c>
+      <c r="F8" s="5" t="n"/>
       <c r="G8" s="5" t="inlineStr">
         <is>
-          <t>0829_patrol_greatwall_916.mov</t>
+          <t>0829_patrol_golddash_916.mov</t>
         </is>
       </c>
       <c r="H8" s="7" t="inlineStr">
@@ -1045,7 +1045,7 @@
       </c>
       <c r="J8" s="6" t="inlineStr">
         <is>
-          <t>Today every pilot flies GREAT WALL: nothing but walls today. Three attempts. Free, in your browser.</t>
+          <t>Today every pilot flies GOLD DASH: Commit the line. The landing is yours. Three attempts. Free, in your browser.</t>
         </is>
       </c>
       <c r="K8" s="5" t="inlineStr">
@@ -1055,18 +1055,18 @@
       </c>
       <c r="L8" s="6" t="inlineStr">
         <is>
-          <t>today every pilot flies great wall: nothing but walls today. three attempts. free, in your browser.</t>
-        </is>
-      </c>
-      <c r="M8" s="6" t="inlineStr"/>
+          <t>today every pilot flies gold dash: commit the line. the landing is yours. three attempts. free, in your browser.</t>
+        </is>
+      </c>
+      <c r="M8" s="6" t="n"/>
       <c r="N8" s="5" t="inlineStr">
         <is>
-          <t>GREAT WALL DAY: Today's ORION Patrol (Day 47)</t>
+          <t>GOLD DASH DAY: Today's ORION Patrol (Day 47)</t>
         </is>
       </c>
       <c r="O8" s="6" t="inlineStr">
         <is>
-          <t>Today's shared seed: GREAT WALL. No ambient drones at all. Only walls, mega walls, and pincers, faster than usual, released to hunt after their sweep. Every pilot flies the same run. Three attempts, free in your browser.
+          <t>Today's shared seed: GOLD DASH. Every pickup is Afterburner. Charge, dash, then one second of invincible arrival. Every pilot flies the same run. Three attempts, free in your browser.
 Play now: https://surviveorion.com
 #dailychallenge #indiegame #browsergame #arcadegame #Shorts</t>
         </is>
@@ -1090,12 +1090,12 @@
       </c>
       <c r="D9" s="5" t="inlineStr">
         <is>
-          <t>PATROL: MAGNETIC FIELD + GIANTS</t>
+          <t>PATROL: BAIT SHOT + YEAR OF THE SERPENT</t>
         </is>
       </c>
       <c r="E9" s="6" t="inlineStr">
         <is>
-          <t>pickups chase you. drones are huge.</t>
+          <t>Pack them, then punch the blob. Every formation slithers today. Watch the trains.</t>
         </is>
       </c>
       <c r="F9" s="5" t="inlineStr">
@@ -1105,7 +1105,7 @@
       </c>
       <c r="G9" s="5" t="inlineStr">
         <is>
-          <t>0830_patrol_magneticfieldgiants_916.mov</t>
+          <t>0830_patrol_baitshotyearoftheserpent_916.mov</t>
         </is>
       </c>
       <c r="H9" s="7" t="inlineStr">
@@ -1120,7 +1120,7 @@
       </c>
       <c r="J9" s="6" t="inlineStr">
         <is>
-          <t>Today every pilot flies MAGNETIC FIELD + GIANTS: pickups chase you. drones are huge. Three attempts. Free, in your browser.</t>
+          <t>Today every pilot flies BAIT SHOT + YEAR OF THE SERPENT: Pack them, then punch the blob. Every formation slithers today. Watch the trains. Three attempts. Free, in your browser.</t>
         </is>
       </c>
       <c r="K9" s="5" t="inlineStr">
@@ -1130,18 +1130,18 @@
       </c>
       <c r="L9" s="6" t="inlineStr">
         <is>
-          <t>today every pilot flies magnetic field + giants: pickups chase you. drones are huge. three attempts. free, in your browser.</t>
-        </is>
-      </c>
-      <c r="M9" s="6" t="inlineStr"/>
+          <t>today every pilot flies bait shot + year of the serpent: pack them, then punch the blob. every formation slithers today. watch the trains. three attempts. free, in your browser.</t>
+        </is>
+      </c>
+      <c r="M9" s="6" t="n"/>
       <c r="N9" s="5" t="inlineStr">
         <is>
-          <t>MAGNETIC FIELD + GIANTS DAY: Today's ORION Patrol (Day 48)</t>
+          <t>BAIT SHOT + YEAR OF THE SERPENT DAY: Today's ORION Patrol (Day 48)</t>
         </is>
       </c>
       <c r="O9" s="6" t="inlineStr">
         <is>
-          <t>Today's shared seed: MAGNETIC FIELD + GIANTS. Pickups slowly drift toward your ship all day. Every drone is bigger and a bit slower, and fewer of them spawn. Every pilot flies the same run. Three attempts, free in your browser.
+          <t>Today's shared seed: BAIT SHOT + YEAR OF THE SERPENT. Only Flares and Pulse Shot drop. The flare does not kill. It gathers a blob. Pulse is the shot. No ambient drones at all. Only serpent trains, more of them, released to hunt after their sweep. Deep in the run the trains keep coming faster and stray drones start leaking in. Every pilot flies the same run. Three attempts, free in your browser.
 Play now: https://surviveorion.com
 #dailychallenge #indiegame #browsergame #arcadegame #Shorts</t>
         </is>
@@ -1165,18 +1165,18 @@
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>STARFALL</t>
+          <t>ION</t>
         </is>
       </c>
       <c r="E10" s="6" t="inlineStr">
         <is>
-          <t>it's raining meteors.</t>
-        </is>
-      </c>
-      <c r="F10" s="5" t="inlineStr"/>
+          <t>Shove the line. Let them break each other.</t>
+        </is>
+      </c>
+      <c r="F10" s="5" t="n"/>
       <c r="G10" s="5" t="inlineStr">
         <is>
-          <t>0831_patrol_starfall_916.mov</t>
+          <t>0831_patrol_ion_916.mov</t>
         </is>
       </c>
       <c r="H10" s="7" t="inlineStr">
@@ -1191,7 +1191,7 @@
       </c>
       <c r="J10" s="6" t="inlineStr">
         <is>
-          <t>Today every pilot flies STARFALL: it's raining meteors. Three attempts. Free, in your browser.</t>
+          <t>Today every pilot flies ION: Shove the line. Let them break each other. Three attempts. Free, in your browser.</t>
         </is>
       </c>
       <c r="K10" s="5" t="inlineStr">
@@ -1201,18 +1201,18 @@
       </c>
       <c r="L10" s="6" t="inlineStr">
         <is>
-          <t>today every pilot flies starfall: it's raining meteors. three attempts. free, in your browser.</t>
-        </is>
-      </c>
-      <c r="M10" s="6" t="inlineStr"/>
+          <t>today every pilot flies ion: shove the line. let them break each other. three attempts. free, in your browser.</t>
+        </is>
+      </c>
+      <c r="M10" s="6" t="n"/>
       <c r="N10" s="5" t="inlineStr">
         <is>
-          <t>STARFALL DAY: Today's ORION Patrol (Day 49)</t>
+          <t>ION DAY: Today's ORION Patrol (Day 49)</t>
         </is>
       </c>
       <c r="O10" s="6" t="inlineStr">
         <is>
-          <t>Today's shared seed: STARFALL. A constant meteor rain falls all run, each impact flashed by a ground reticle first. The only drop is Shield, a little more often. Every pilot flies the same run. Three attempts, free in your browser.
+          <t>Today's shared seed: ION. Every pickup is Ion. A forward shockwave pushes drones. The pushed ones live. What they slam dies. Every pilot flies the same run. Three attempts, free in your browser.
 Play now: https://surviveorion.com
 #dailychallenge #indiegame #browsergame #arcadegame #Shorts</t>
         </is>
@@ -1236,18 +1236,18 @@
       </c>
       <c r="D11" s="5" t="inlineStr">
         <is>
-          <t>BLACKOUT</t>
+          <t>STARFALL</t>
         </is>
       </c>
       <c r="E11" s="6" t="inlineStr">
         <is>
-          <t>half the warning today.</t>
-        </is>
-      </c>
-      <c r="F11" s="5" t="inlineStr"/>
+          <t>The sky opens early. Shields are scarce.</t>
+        </is>
+      </c>
+      <c r="F11" s="5" t="n"/>
       <c r="G11" s="5" t="inlineStr">
         <is>
-          <t>0901_patrol_blackout_916.mov</t>
+          <t>0901_patrol_starfall_916.mov</t>
         </is>
       </c>
       <c r="H11" s="7" t="inlineStr">
@@ -1262,7 +1262,7 @@
       </c>
       <c r="J11" s="6" t="inlineStr">
         <is>
-          <t>Today every pilot flies BLACKOUT: half the warning today. Three attempts. Free, in your browser.</t>
+          <t>Today every pilot flies STARFALL: The sky opens early. Shields are scarce. Three attempts. Free, in your browser.</t>
         </is>
       </c>
       <c r="K11" s="5" t="inlineStr">
@@ -1272,18 +1272,18 @@
       </c>
       <c r="L11" s="6" t="inlineStr">
         <is>
-          <t>today every pilot flies blackout: half the warning today. three attempts. free, in your browser.</t>
-        </is>
-      </c>
-      <c r="M11" s="6" t="inlineStr"/>
+          <t>today every pilot flies starfall: the sky opens early. shields are scarce. three attempts. free, in your browser.</t>
+        </is>
+      </c>
+      <c r="M11" s="6" t="n"/>
       <c r="N11" s="5" t="inlineStr">
         <is>
-          <t>BLACKOUT DAY: Today's ORION Patrol (Day 50)</t>
+          <t>STARFALL DAY: Today's ORION Patrol (Day 50)</t>
         </is>
       </c>
       <c r="O11" s="6" t="inlineStr">
         <is>
-          <t>Today's shared seed: BLACKOUT. On-screen spawn warnings are much shorter (0.5s instead of 1.4s). Everything else is normal. Every pilot flies the same run. Three attempts, free in your browser.
+          <t>Today's shared seed: STARFALL. Meteor rain from the first seconds. Shield is the only drop, and it is late. Every pilot flies the same run. Three attempts, free in your browser.
 Play now: https://surviveorion.com
 #dailychallenge #indiegame #browsergame #arcadegame #Shorts</t>
         </is>
@@ -1307,18 +1307,18 @@
       </c>
       <c r="D12" s="5" t="inlineStr">
         <is>
-          <t>CRYO WINTER</t>
+          <t>RED ALERT</t>
         </is>
       </c>
       <c r="E12" s="6" t="inlineStr">
         <is>
-          <t>everything you grab freezes.</t>
-        </is>
-      </c>
-      <c r="F12" s="5" t="inlineStr"/>
+          <t>Klaxons up. Everything moves faster except you.</t>
+        </is>
+      </c>
+      <c r="F12" s="5" t="n"/>
       <c r="G12" s="5" t="inlineStr">
         <is>
-          <t>0902_patrol_cryowinter_916.mov</t>
+          <t>0902_patrol_redalert_916.mov</t>
         </is>
       </c>
       <c r="H12" s="7" t="inlineStr">
@@ -1333,7 +1333,7 @@
       </c>
       <c r="J12" s="6" t="inlineStr">
         <is>
-          <t>Today every pilot flies CRYO WINTER: everything you grab freezes. Three attempts. Free, in your browser.</t>
+          <t>Today every pilot flies RED ALERT: Klaxons up. Everything moves faster except you. Three attempts. Free, in your browser.</t>
         </is>
       </c>
       <c r="K12" s="5" t="inlineStr">
@@ -1343,18 +1343,18 @@
       </c>
       <c r="L12" s="6" t="inlineStr">
         <is>
-          <t>today every pilot flies cryo winter: everything you grab freezes. three attempts. free, in your browser.</t>
-        </is>
-      </c>
-      <c r="M12" s="6" t="inlineStr"/>
+          <t>today every pilot flies red alert: klaxons up. everything moves faster except you. three attempts. free, in your browser.</t>
+        </is>
+      </c>
+      <c r="M12" s="6" t="n"/>
       <c r="N12" s="5" t="inlineStr">
         <is>
-          <t>CRYO WINTER DAY: Today's ORION Patrol (Day 51)</t>
+          <t>RED ALERT DAY: Today's ORION Patrol (Day 51)</t>
         </is>
       </c>
       <c r="O12" s="6" t="inlineStr">
         <is>
-          <t>Today's shared seed: CRYO WINTER. Every pickup is a Cryo Field. Every pilot flies the same run. Three attempts, free in your browser.
+          <t>Today's shared seed: RED ALERT. Spawn rate, formation frequency, and pickup drops all sped up. Drone speed is unchanged. Every pilot flies the same run. Three attempts, free in your browser.
 Play now: https://surviveorion.com
 #dailychallenge #indiegame #browsergame #arcadegame #Shorts</t>
         </is>
@@ -1449,18 +1449,18 @@
       </c>
       <c r="D14" s="5" t="inlineStr">
         <is>
-          <t>HUNTING PARTY</t>
+          <t>THE FLOOD</t>
         </is>
       </c>
       <c r="E14" s="6" t="inlineStr">
         <is>
-          <t>the hunters are coordinated today.</t>
-        </is>
-      </c>
-      <c r="F14" s="5" t="inlineStr"/>
+          <t>No formations. They just keep popping in.</t>
+        </is>
+      </c>
+      <c r="F14" s="5" t="n"/>
       <c r="G14" s="5" t="inlineStr">
         <is>
-          <t>0903_patrol_huntingparty_916.mov</t>
+          <t>0903_patrol_theflood_916.mov</t>
         </is>
       </c>
       <c r="H14" s="7" t="inlineStr">
@@ -1475,7 +1475,7 @@
       </c>
       <c r="J14" s="6" t="inlineStr">
         <is>
-          <t>Today every pilot flies HUNTING PARTY: the hunters are coordinated today. Three attempts. Free, in your browser.</t>
+          <t>Today every pilot flies THE FLOOD: No formations. They just keep popping in. Three attempts. Free, in your browser.</t>
         </is>
       </c>
       <c r="K14" s="5" t="inlineStr">
@@ -1485,18 +1485,18 @@
       </c>
       <c r="L14" s="6" t="inlineStr">
         <is>
-          <t>today every pilot flies hunting party: the hunters are coordinated today. three attempts. free, in your browser.</t>
-        </is>
-      </c>
-      <c r="M14" s="6" t="inlineStr"/>
+          <t>today every pilot flies the flood: no formations. they just keep popping in. three attempts. free, in your browser.</t>
+        </is>
+      </c>
+      <c r="M14" s="6" t="n"/>
       <c r="N14" s="5" t="inlineStr">
         <is>
-          <t>HUNTING PARTY DAY: Today's ORION Patrol (Day 52)</t>
+          <t>THE FLOOD DAY: Today's ORION Patrol (Day 52)</t>
         </is>
       </c>
       <c r="O14" s="6" t="inlineStr">
         <is>
-          <t>Today's shared seed: HUNTING PARTY. Waves of hunters close in from different edges and converge, growing in size and frequency fast after the first wave. Every pilot flies the same run. Three attempts, free in your browser.
+          <t>Today's shared seed: THE FLOOD. A constant beat from the edges. The beat speeds up the whole run. Every pilot flies the same run. Three attempts, free in your browser.
 Play now: https://surviveorion.com
 #dailychallenge #indiegame #browsergame #arcadegame #Shorts</t>
         </is>
@@ -1520,18 +1520,18 @@
       </c>
       <c r="D15" s="5" t="inlineStr">
         <is>
-          <t>DEMOLITION DAY</t>
+          <t>THUNDER</t>
         </is>
       </c>
       <c r="E15" s="6" t="inlineStr">
         <is>
-          <t>bombs. nonstop.</t>
-        </is>
-      </c>
-      <c r="F15" s="5" t="inlineStr"/>
+          <t>Aim the ray. Let it hop.</t>
+        </is>
+      </c>
+      <c r="F15" s="5" t="n"/>
       <c r="G15" s="5" t="inlineStr">
         <is>
-          <t>0904_patrol_demolitionday_916.mov</t>
+          <t>0904_patrol_thunder_916.mov</t>
         </is>
       </c>
       <c r="H15" s="7" t="inlineStr">
@@ -1546,7 +1546,7 @@
       </c>
       <c r="J15" s="6" t="inlineStr">
         <is>
-          <t>Today every pilot flies DEMOLITION DAY: bombs. nonstop. Three attempts. Free, in your browser.</t>
+          <t>Today every pilot flies THUNDER: Aim the ray. Let it hop. Three attempts. Free, in your browser.</t>
         </is>
       </c>
       <c r="K15" s="5" t="inlineStr">
@@ -1556,18 +1556,18 @@
       </c>
       <c r="L15" s="6" t="inlineStr">
         <is>
-          <t>today every pilot flies demolition day: bombs. nonstop. three attempts. free, in your browser.</t>
-        </is>
-      </c>
-      <c r="M15" s="6" t="inlineStr"/>
+          <t>today every pilot flies thunder: aim the ray. let it hop. three attempts. free, in your browser.</t>
+        </is>
+      </c>
+      <c r="M15" s="6" t="n"/>
       <c r="N15" s="5" t="inlineStr">
         <is>
-          <t>DEMOLITION DAY DAY: Today's ORION Patrol (Day 53)</t>
+          <t>THUNDER DAY: Today's ORION Patrol (Day 53)</t>
         </is>
       </c>
       <c r="O15" s="6" t="inlineStr">
         <is>
-          <t>Today's shared seed: DEMOLITION DAY. Bomb slabs deploy continuously and detonate into shrapnel, crowding the space fast after the first minute. Every pilot flies the same run. Three attempts, free in your browser.
+          <t>Today's shared seed: THUNDER. Every pickup is Thunder. A lightning ray along your nose. Each kill sparks Arc hops. Ray kills pay double. Every pilot flies the same run. Three attempts, free in your browser.
 Play now: https://surviveorion.com
 #dailychallenge #indiegame #browsergame #arcadegame #Shorts</t>
         </is>
@@ -1662,18 +1662,18 @@
       </c>
       <c r="D17" s="5" t="inlineStr">
         <is>
-          <t>GIANTS</t>
+          <t>YEAR OF THE SERPENT</t>
         </is>
       </c>
       <c r="E17" s="6" t="inlineStr">
         <is>
-          <t>every drone is huge today.</t>
-        </is>
-      </c>
-      <c r="F17" s="5" t="inlineStr"/>
+          <t>Every formation slithers today. Watch the trains.</t>
+        </is>
+      </c>
+      <c r="F17" s="5" t="n"/>
       <c r="G17" s="5" t="inlineStr">
         <is>
-          <t>0905_patrol_giants_916.mov</t>
+          <t>0905_patrol_yearoftheserpent_916.mov</t>
         </is>
       </c>
       <c r="H17" s="7" t="inlineStr">
@@ -1688,7 +1688,7 @@
       </c>
       <c r="J17" s="6" t="inlineStr">
         <is>
-          <t>Today every pilot flies GIANTS: every drone is huge today. Three attempts. Free, in your browser.</t>
+          <t>Today every pilot flies YEAR OF THE SERPENT: Every formation slithers today. Watch the trains. Three attempts. Free, in your browser.</t>
         </is>
       </c>
       <c r="K17" s="5" t="inlineStr">
@@ -1698,18 +1698,18 @@
       </c>
       <c r="L17" s="6" t="inlineStr">
         <is>
-          <t>today every pilot flies giants: every drone is huge today. three attempts. free, in your browser.</t>
-        </is>
-      </c>
-      <c r="M17" s="6" t="inlineStr"/>
+          <t>today every pilot flies year of the serpent: every formation slithers today. watch the trains. three attempts. free, in your browser.</t>
+        </is>
+      </c>
+      <c r="M17" s="6" t="n"/>
       <c r="N17" s="5" t="inlineStr">
         <is>
-          <t>GIANTS DAY: Today's ORION Patrol (Day 54)</t>
+          <t>YEAR OF THE SERPENT DAY: Today's ORION Patrol (Day 54)</t>
         </is>
       </c>
       <c r="O17" s="6" t="inlineStr">
         <is>
-          <t>Today's shared seed: GIANTS. Every drone is bigger and a bit slower. Fewer of them spawn. Every pilot flies the same run. Three attempts, free in your browser.
+          <t>Today's shared seed: YEAR OF THE SERPENT. No ambient drones at all. Only serpent trains, more of them, released to hunt after their sweep. Deep in the run the trains keep coming faster and stray drones start leaking in. Every pilot flies the same run. Three attempts, free in your browser.
 Play now: https://surviveorion.com
 #dailychallenge #indiegame #browsergame #arcadegame #Shorts</t>
         </is>
@@ -1733,12 +1733,12 @@
       </c>
       <c r="D18" s="5" t="inlineStr">
         <is>
-          <t>PATROL: ARSENAL + HUNTING PARTY</t>
+          <t>PATROL: MAGNETIC FIELD + CLOAK</t>
         </is>
       </c>
       <c r="E18" s="6" t="inlineStr">
         <is>
-          <t>double drops. coordinated hunters.</t>
+          <t>The pickups want to find you today. They lose the lock. You seed the dark.</t>
         </is>
       </c>
       <c r="F18" s="5" t="inlineStr">
@@ -1748,7 +1748,7 @@
       </c>
       <c r="G18" s="5" t="inlineStr">
         <is>
-          <t>0906_patrol_arsenalhuntingparty_916.mov</t>
+          <t>0906_patrol_magneticfieldcloak_916.mov</t>
         </is>
       </c>
       <c r="H18" s="7" t="inlineStr">
@@ -1763,7 +1763,7 @@
       </c>
       <c r="J18" s="6" t="inlineStr">
         <is>
-          <t>Today every pilot flies ARSENAL + HUNTING PARTY: double drops. coordinated hunters. Three attempts. Free, in your browser.</t>
+          <t>Today every pilot flies MAGNETIC FIELD + CLOAK: The pickups want to find you today. They lose the lock. You seed the dark. Three attempts. Free, in your browser.</t>
         </is>
       </c>
       <c r="K18" s="5" t="inlineStr">
@@ -1773,18 +1773,18 @@
       </c>
       <c r="L18" s="6" t="inlineStr">
         <is>
-          <t>today every pilot flies arsenal + hunting party: double drops. coordinated hunters. three attempts. free, in your browser.</t>
-        </is>
-      </c>
-      <c r="M18" s="6" t="inlineStr"/>
+          <t>today every pilot flies magnetic field + cloak: the pickups want to find you today. they lose the lock. you seed the dark. three attempts. free, in your browser.</t>
+        </is>
+      </c>
+      <c r="M18" s="6" t="n"/>
       <c r="N18" s="5" t="inlineStr">
         <is>
-          <t>ARSENAL + HUNTING PARTY DAY: Today's ORION Patrol (Day 55)</t>
+          <t>MAGNETIC FIELD + CLOAK DAY: Today's ORION Patrol (Day 55)</t>
         </is>
       </c>
       <c r="O18" s="6" t="inlineStr">
         <is>
-          <t>Today's shared seed: ARSENAL + HUNTING PARTY. Pickup drops roughly twice as often. Waves of hunters close in from different edges and converge, growing fast after the first wave. Every pilot flies the same run. Three attempts, free in your browser.
+          <t>Today's shared seed: MAGNETIC FIELD + CLOAK. Pickups slowly drift toward your ship all day, on top of their normal wander. Every pickup is Cloak. Drones hover, lost. Invisible bombs drop along your path and explode when you reappear. Every pilot flies the same run. Three attempts, free in your browser.
 Play now: https://surviveorion.com
 #dailychallenge #indiegame #browsergame #arcadegame #Shorts</t>
         </is>
@@ -1879,18 +1879,18 @@
       </c>
       <c r="D20" s="5" t="inlineStr">
         <is>
-          <t>THE FLOOD</t>
+          <t>RAM RAID</t>
         </is>
       </c>
       <c r="E20" s="6" t="inlineStr">
         <is>
-          <t>the swarm never stops.</t>
-        </is>
-      </c>
-      <c r="F20" s="5" t="inlineStr"/>
+          <t>The shell is short. Spend it, then dodge naked.</t>
+        </is>
+      </c>
+      <c r="F20" s="5" t="n"/>
       <c r="G20" s="5" t="inlineStr">
         <is>
-          <t>0907_patrol_theflood_916.mov</t>
+          <t>0907_patrol_ramraid_916.mov</t>
         </is>
       </c>
       <c r="H20" s="7" t="inlineStr">
@@ -1905,7 +1905,7 @@
       </c>
       <c r="J20" s="6" t="inlineStr">
         <is>
-          <t>Today every pilot flies THE FLOOD: the swarm never stops. Three attempts. Free, in your browser.</t>
+          <t>Today every pilot flies RAM RAID: The shell is short. Spend it, then dodge naked. Three attempts. Free, in your browser.</t>
         </is>
       </c>
       <c r="K20" s="5" t="inlineStr">
@@ -1915,18 +1915,18 @@
       </c>
       <c r="L20" s="6" t="inlineStr">
         <is>
-          <t>today every pilot flies the flood: the swarm never stops. three attempts. free, in your browser.</t>
-        </is>
-      </c>
-      <c r="M20" s="6" t="inlineStr"/>
+          <t>today every pilot flies ram raid: the shell is short. spend it, then dodge naked. three attempts. free, in your browser.</t>
+        </is>
+      </c>
+      <c r="M20" s="6" t="n"/>
       <c r="N20" s="5" t="inlineStr">
         <is>
-          <t>THE FLOOD DAY: Today's ORION Patrol (Day 56)</t>
+          <t>RAM RAID DAY: Today's ORION Patrol (Day 56)</t>
         </is>
       </c>
       <c r="O20" s="6" t="inlineStr">
         <is>
-          <t>Today's shared seed: THE FLOOD. Formations almost never happen. Ambient density is up, but arrives in clearer packs with lanes between them. Every pilot flies the same run. Three attempts, free in your browser.
+          <t>Today's shared seed: RAM RAID. Starshell is the only drop, and it is scarce. The shell lasts about two seconds. You are invincible while it is up. Every pilot flies the same run. Three attempts, free in your browser.
 Play now: https://surviveorion.com
 #dailychallenge #indiegame #browsergame #arcadegame #Shorts</t>
         </is>
@@ -1950,18 +1950,18 @@
       </c>
       <c r="D21" s="5" t="inlineStr">
         <is>
-          <t>WHEELHOUSE</t>
+          <t>SINGULARITY</t>
         </is>
       </c>
       <c r="E21" s="6" t="inlineStr">
         <is>
-          <t>dodge the traffic today.</t>
-        </is>
-      </c>
-      <c r="F21" s="5" t="inlineStr"/>
+          <t>The banned singularity is back for one day. Use it well.</t>
+        </is>
+      </c>
+      <c r="F21" s="5" t="n"/>
       <c r="G21" s="5" t="inlineStr">
         <is>
-          <t>0908_patrol_wheelhouse_916.mov</t>
+          <t>0908_patrol_singularity_916.mov</t>
         </is>
       </c>
       <c r="H21" s="7" t="inlineStr">
@@ -1976,7 +1976,7 @@
       </c>
       <c r="J21" s="6" t="inlineStr">
         <is>
-          <t>Today every pilot flies WHEELHOUSE: dodge the traffic today. Three attempts. Free, in your browser.</t>
+          <t>Today every pilot flies SINGULARITY: The banned singularity is back for one day. Use it well. Three attempts. Free, in your browser.</t>
         </is>
       </c>
       <c r="K21" s="5" t="inlineStr">
@@ -1986,18 +1986,18 @@
       </c>
       <c r="L21" s="6" t="inlineStr">
         <is>
-          <t>today every pilot flies wheelhouse: dodge the traffic today. three attempts. free, in your browser.</t>
-        </is>
-      </c>
-      <c r="M21" s="6" t="inlineStr"/>
+          <t>today every pilot flies singularity: the banned singularity is back for one day. use it well. three attempts. free, in your browser.</t>
+        </is>
+      </c>
+      <c r="M21" s="6" t="n"/>
       <c r="N21" s="5" t="inlineStr">
         <is>
-          <t>WHEELHOUSE DAY: Today's ORION Patrol (Day 57)</t>
+          <t>SINGULARITY DAY: Today's ORION Patrol (Day 57)</t>
         </is>
       </c>
       <c r="O21" s="6" t="inlineStr">
         <is>
-          <t>Today's shared seed: WHEELHOUSE. Wheels roll through in lanes from alternating sides, Frogger-style. One lane at the open, then rush hour builds fast. Every pilot flies the same run. Three attempts, free in your browser.
+          <t>Today's shared seed: SINGULARITY. Vortex (normally benched) drops often today. Every pilot flies the same run. Three attempts, free in your browser.
 Play now: https://surviveorion.com
 #dailychallenge #indiegame #browsergame #arcadegame #Shorts</t>
         </is>

</xml_diff>

<commit_message>
Move GREAT WALL Buffer posts to the next real patrol day. [skip render]
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/ORION_Publishing_Calendar.xlsx
+++ b/ORION_Publishing_Calendar.xlsx
@@ -482,7 +482,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O21"/>
+  <dimension ref="A1:O22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -2003,6 +2003,75 @@
         </is>
       </c>
     </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Sat</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>TODAY'S PATROL</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>GREAT WALL</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>nothing but walls today.</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>0827_greatwall_916.mov</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>Linked</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>Scheduled</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>Today every pilot flies GREAT WALL: nothing but walls today. Three attempts. Free, in your browser.</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>#dailychallenge #indiegame #browsergame #arcadegame</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>today every pilot flies great wall: nothing but walls today. three attempts. free, in your browser.</t>
+        </is>
+      </c>
+      <c r="N22" t="inlineStr">
+        <is>
+          <t>GREAT WALL DAY: Today's ORION Patrol (Day 75)</t>
+        </is>
+      </c>
+      <c r="O22" t="inlineStr">
+        <is>
+          <t>Today's shared seed: GREAT WALL. No ambient drones at all. Only walls, mega walls, and pincers, faster than usual, released to hunt after their sweep. Every pilot flies the same run. Three attempts, free in your browser.
+Play now: https://surviveorion.com
+#dailychallenge #indiegame #browsergame #arcadegame #Shorts</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Host four new Orion finals and add the Nature's Call calendar slot.
Buffer needs public H.264 URLs; GOLD DASH copy now matches the live briefing.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/ORION_Publishing_Calendar.xlsx
+++ b/ORION_Publishing_Calendar.xlsx
@@ -16,7 +16,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
+  </numFmts>
   <fonts count="5">
     <font>
       <name val="Calibri"/>
@@ -94,7 +96,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -115,6 +117,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
     </xf>
   </cellXfs>
@@ -482,7 +487,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O22"/>
+  <dimension ref="A1:O24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -959,17 +964,17 @@
       <c r="F7" s="5" t="inlineStr"/>
       <c r="G7" s="5" t="inlineStr">
         <is>
-          <t>0829_ratethisdodge_916.mov</t>
+          <t>0828_ratemydodge_916.mp4</t>
         </is>
       </c>
       <c r="H7" s="7" t="inlineStr">
         <is>
-          <t>Not linked yet</t>
+          <t>Linked</t>
         </is>
       </c>
       <c r="I7" s="5" t="inlineStr">
         <is>
-          <t>Draft</t>
+          <t>Approved</t>
         </is>
       </c>
       <c r="J7" s="6" t="inlineStr">
@@ -1024,28 +1029,28 @@
       </c>
       <c r="E8" s="6" t="inlineStr">
         <is>
-          <t>Commit the line. The landing is yours.</t>
+          <t>Stop, point, burn the line.</t>
         </is>
       </c>
       <c r="F8" s="5" t="n"/>
       <c r="G8" s="5" t="inlineStr">
         <is>
-          <t>0829_patrol_golddash_916.mov</t>
+          <t>0828_GOLDDASH_916.mp4</t>
         </is>
       </c>
       <c r="H8" s="7" t="inlineStr">
         <is>
-          <t>Not linked yet</t>
+          <t>Linked</t>
         </is>
       </c>
       <c r="I8" s="5" t="inlineStr">
         <is>
-          <t>Draft</t>
+          <t>Approved</t>
         </is>
       </c>
       <c r="J8" s="6" t="inlineStr">
         <is>
-          <t>Today every pilot flies GOLD DASH: Commit the line. The landing is yours. Three attempts. Free, in your browser.</t>
+          <t>Today every pilot flies GOLD DASH: Stop, point, burn the line. Three attempts. Free, in your browser.</t>
         </is>
       </c>
       <c r="K8" s="5" t="inlineStr">
@@ -1055,7 +1060,7 @@
       </c>
       <c r="L8" s="6" t="inlineStr">
         <is>
-          <t>today every pilot flies gold dash: commit the line. the landing is yours. three attempts. free, in your browser.</t>
+          <t>today every pilot flies gold dash: stop, point, burn the line. three attempts. free, in your browser.</t>
         </is>
       </c>
       <c r="M8" s="6" t="n"/>
@@ -1066,17 +1071,15 @@
       </c>
       <c r="O8" s="6" t="inlineStr">
         <is>
-          <t>Today's shared seed: GOLD DASH. Every pickup is Afterburner. Charge, dash, then one second of invincible arrival. Every pilot flies the same run. Three attempts, free in your browser.
+          <t>Today's shared seed: GOLD DASH. Every pickup is Afterburner. Grab one and you freeze, aim, then dash. You ram while aiming and the corridor burns. Another dash always waits across the field. Every pilot flies the same run. Three attempts, free in your browser.
 Play now: https://surviveorion.com
 #dailychallenge #indiegame #browsergame #arcadegame #Shorts</t>
         </is>
       </c>
     </row>
     <row r="9" ht="60" customHeight="1">
-      <c r="A9" s="5" t="inlineStr">
-        <is>
-          <t>2026-08-30</t>
-        </is>
+      <c r="A9" s="8" t="n">
+        <v>46264</v>
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
@@ -1085,61 +1088,132 @@
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>TODAY'S PATROL · SUNDAY DOUBLE</t>
+          <t>POV</t>
         </is>
       </c>
       <c r="D9" s="5" t="inlineStr">
         <is>
-          <t>PATROL: BAIT SHOT + YEAR OF THE SERPENT</t>
+          <t>Nature's Call</t>
         </is>
       </c>
       <c r="E9" s="6" t="inlineStr">
         <is>
-          <t>Pack them, then punch the blob. Every formation slithers today. Watch the trains.</t>
-        </is>
-      </c>
-      <c r="F9" s="5" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
+          <t>POV: answering nature's call while trying to survive</t>
+        </is>
+      </c>
+      <c r="F9" s="5" t="n"/>
       <c r="G9" s="5" t="inlineStr">
         <is>
-          <t>0830_patrol_baitshotyearoftheserpent_916.mov</t>
+          <t>0828_naturecall_916.mp4</t>
         </is>
       </c>
       <c r="H9" s="7" t="inlineStr">
         <is>
-          <t>Not linked yet</t>
+          <t>Linked</t>
         </is>
       </c>
       <c r="I9" s="5" t="inlineStr">
         <is>
-          <t>Draft</t>
+          <t>Approved</t>
         </is>
       </c>
       <c r="J9" s="6" t="inlineStr">
         <is>
-          <t>Today every pilot flies BAIT SHOT + YEAR OF THE SERPENT: Pack them, then punch the blob. Every formation slithers today. Watch the trains. Three attempts. Free, in your browser.</t>
+          <t>POV: answering nature's call while trying to survive 💀 4x speed. Three attempts. Free browser game, link in bio.</t>
         </is>
       </c>
       <c r="K9" s="5" t="inlineStr">
         <is>
-          <t>#dailychallenge #indiegame #browsergame #arcadegame</t>
+          <t>#gamingmemes #indiegame #fail #dailychallenge #browsergame</t>
         </is>
       </c>
       <c r="L9" s="6" t="inlineStr">
         <is>
-          <t>today every pilot flies bait shot + year of the serpent: pack them, then punch the blob. every formation slithers today. watch the trains. three attempts. free, in your browser.</t>
+          <t>pov: answering nature's call while trying to survive 💀 free daily dodge game, 3 attempts, link in bio</t>
         </is>
       </c>
       <c r="M9" s="6" t="n"/>
       <c r="N9" s="5" t="inlineStr">
         <is>
+          <t>POV: Answering Nature's Call While Trying to Survive (ORION)</t>
+        </is>
+      </c>
+      <c r="O9" s="6" t="inlineStr">
+        <is>
+          <t>4x speed. Same swarm. Nature called anyway. Free daily dodging game, three attempts a day.
+Play: https://surviveorion.com
+#gamingmemes #indiegame #Shorts</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="60" customHeight="1">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>Sun</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>TODAY'S PATROL · SUNDAY DOUBLE</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="inlineStr">
+        <is>
+          <t>PATROL: BAIT SHOT + YEAR OF THE SERPENT</t>
+        </is>
+      </c>
+      <c r="E10" s="6" t="inlineStr">
+        <is>
+          <t>Pack them, then punch the blob. Every formation slithers today. Watch the trains.</t>
+        </is>
+      </c>
+      <c r="F10" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G10" s="5" t="inlineStr">
+        <is>
+          <t>0830_patrol_baitshotyearoftheserpent_916.mov</t>
+        </is>
+      </c>
+      <c r="H10" s="7" t="inlineStr">
+        <is>
+          <t>Not linked yet</t>
+        </is>
+      </c>
+      <c r="I10" s="5" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="J10" s="6" t="inlineStr">
+        <is>
+          <t>Today every pilot flies BAIT SHOT + YEAR OF THE SERPENT: Pack them, then punch the blob. Every formation slithers today. Watch the trains. Three attempts. Free, in your browser.</t>
+        </is>
+      </c>
+      <c r="K10" s="5" t="inlineStr">
+        <is>
+          <t>#dailychallenge #indiegame #browsergame #arcadegame</t>
+        </is>
+      </c>
+      <c r="L10" s="6" t="inlineStr">
+        <is>
+          <t>today every pilot flies bait shot + year of the serpent: pack them, then punch the blob. every formation slithers today. watch the trains. three attempts. free, in your browser.</t>
+        </is>
+      </c>
+      <c r="M10" s="6" t="n"/>
+      <c r="N10" s="5" t="inlineStr">
+        <is>
           <t>BAIT SHOT + YEAR OF THE SERPENT DAY: Today's ORION Patrol (Day 48)</t>
         </is>
       </c>
-      <c r="O9" s="6" t="inlineStr">
+      <c r="O10" s="6" t="inlineStr">
         <is>
           <t>Today's shared seed: BAIT SHOT + YEAR OF THE SERPENT. Only Flares and Pulse Shot drop. The flare does not kill. It gathers a blob. Pulse is the shot. No ambient drones at all. Only serpent trains, more of them, released to hunt after their sweep. Deep in the run the trains keep coming faster and stray drones start leaking in. Every pilot flies the same run. Three attempts, free in your browser.
 Play now: https://surviveorion.com
@@ -1147,70 +1221,139 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="60" customHeight="1">
-      <c r="A10" s="5" t="inlineStr">
+    <row r="11" ht="60" customHeight="1">
+      <c r="A11" s="8" t="n">
+        <v>46265</v>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>Mon</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>SPACE DUST</t>
+        </is>
+      </c>
+      <c r="D11" s="5" t="inlineStr">
+        <is>
+          <t>Space Dust</t>
+        </is>
+      </c>
+      <c r="E11" s="6" t="inlineStr">
+        <is>
+          <t>speedrun to the afterlife</t>
+        </is>
+      </c>
+      <c r="F11" s="5" t="n"/>
+      <c r="G11" s="5" t="inlineStr">
+        <is>
+          <t>0828_spacedust_916.mp4</t>
+        </is>
+      </c>
+      <c r="H11" s="7" t="inlineStr">
+        <is>
+          <t>Linked</t>
+        </is>
+      </c>
+      <c r="I11" s="5" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="J11" s="6" t="inlineStr">
+        <is>
+          <t>speedrun to the afterlife 💀 The daily patrol remains undefeated. Free browser game, link in bio.</t>
+        </is>
+      </c>
+      <c r="K11" s="5" t="inlineStr">
+        <is>
+          <t>#gamingmemes #indiegame #fail #dailychallenge #browsergame</t>
+        </is>
+      </c>
+      <c r="L11" s="6" t="inlineStr">
+        <is>
+          <t>speedrun to the afterlife 💀 free daily dodge game, 3 attempts, new run every day, link in bio</t>
+        </is>
+      </c>
+      <c r="M11" s="6" t="n"/>
+      <c r="N11" s="5" t="inlineStr">
+        <is>
+          <t>Speedrun to the Afterlife (ORION Space Dust)</t>
+        </is>
+      </c>
+      <c r="O11" s="6" t="inlineStr">
+        <is>
+          <t>The daily patrol is undefeated. Free dodging game, same run for every pilot.
+Play: https://surviveorion.com
+#Shorts</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="60" customHeight="1">
+      <c r="A12" s="5" t="inlineStr">
         <is>
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="B10" s="5" t="inlineStr">
+      <c r="B12" s="5" t="inlineStr">
         <is>
           <t>Mon</t>
         </is>
       </c>
-      <c r="C10" s="5" t="inlineStr">
+      <c r="C12" s="5" t="inlineStr">
         <is>
           <t>TODAY'S PATROL</t>
         </is>
       </c>
-      <c r="D10" s="5" t="inlineStr">
+      <c r="D12" s="5" t="inlineStr">
         <is>
           <t>ION</t>
         </is>
       </c>
-      <c r="E10" s="6" t="inlineStr">
+      <c r="E12" s="6" t="inlineStr">
         <is>
           <t>Shove the line. Let them break each other.</t>
         </is>
       </c>
-      <c r="F10" s="5" t="n"/>
-      <c r="G10" s="5" t="inlineStr">
+      <c r="F12" s="5" t="n"/>
+      <c r="G12" s="5" t="inlineStr">
         <is>
           <t>0831_patrol_ion_916.mov</t>
         </is>
       </c>
-      <c r="H10" s="7" t="inlineStr">
+      <c r="H12" s="7" t="inlineStr">
         <is>
           <t>Not linked yet</t>
         </is>
       </c>
-      <c r="I10" s="5" t="inlineStr">
+      <c r="I12" s="5" t="inlineStr">
         <is>
           <t>Draft</t>
         </is>
       </c>
-      <c r="J10" s="6" t="inlineStr">
+      <c r="J12" s="6" t="inlineStr">
         <is>
           <t>Today every pilot flies ION: Shove the line. Let them break each other. Three attempts. Free, in your browser.</t>
         </is>
       </c>
-      <c r="K10" s="5" t="inlineStr">
+      <c r="K12" s="5" t="inlineStr">
         <is>
           <t>#dailychallenge #indiegame #browsergame #arcadegame</t>
         </is>
       </c>
-      <c r="L10" s="6" t="inlineStr">
+      <c r="L12" s="6" t="inlineStr">
         <is>
           <t>today every pilot flies ion: shove the line. let them break each other. three attempts. free, in your browser.</t>
         </is>
       </c>
-      <c r="M10" s="6" t="n"/>
-      <c r="N10" s="5" t="inlineStr">
+      <c r="M12" s="6" t="n"/>
+      <c r="N12" s="5" t="inlineStr">
         <is>
           <t>ION DAY: Today's ORION Patrol (Day 49)</t>
         </is>
       </c>
-      <c r="O10" s="6" t="inlineStr">
+      <c r="O12" s="6" t="inlineStr">
         <is>
           <t>Today's shared seed: ION. Every pickup is Ion. A forward shockwave pushes drones. The pushed ones live. What they slam dies. Every pilot flies the same run. Three attempts, free in your browser.
 Play now: https://surviveorion.com
@@ -1218,70 +1361,70 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="60" customHeight="1">
-      <c r="A11" s="5" t="inlineStr">
+    <row r="13" ht="60" customHeight="1">
+      <c r="A13" s="5" t="inlineStr">
         <is>
           <t>2026-09-01</t>
         </is>
       </c>
-      <c r="B11" s="5" t="inlineStr">
+      <c r="B13" s="5" t="inlineStr">
         <is>
           <t>Tue</t>
         </is>
       </c>
-      <c r="C11" s="5" t="inlineStr">
+      <c r="C13" s="5" t="inlineStr">
         <is>
           <t>TODAY'S PATROL</t>
         </is>
       </c>
-      <c r="D11" s="5" t="inlineStr">
+      <c r="D13" s="5" t="inlineStr">
         <is>
           <t>STARFALL</t>
         </is>
       </c>
-      <c r="E11" s="6" t="inlineStr">
+      <c r="E13" s="6" t="inlineStr">
         <is>
           <t>The sky opens early. Shields are scarce.</t>
         </is>
       </c>
-      <c r="F11" s="5" t="n"/>
-      <c r="G11" s="5" t="inlineStr">
+      <c r="F13" s="5" t="n"/>
+      <c r="G13" s="5" t="inlineStr">
         <is>
           <t>0901_patrol_starfall_916.mov</t>
         </is>
       </c>
-      <c r="H11" s="7" t="inlineStr">
+      <c r="H13" s="7" t="inlineStr">
         <is>
           <t>Not linked yet</t>
         </is>
       </c>
-      <c r="I11" s="5" t="inlineStr">
+      <c r="I13" s="5" t="inlineStr">
         <is>
           <t>Draft</t>
         </is>
       </c>
-      <c r="J11" s="6" t="inlineStr">
+      <c r="J13" s="6" t="inlineStr">
         <is>
           <t>Today every pilot flies STARFALL: The sky opens early. Shields are scarce. Three attempts. Free, in your browser.</t>
         </is>
       </c>
-      <c r="K11" s="5" t="inlineStr">
+      <c r="K13" s="5" t="inlineStr">
         <is>
           <t>#dailychallenge #indiegame #browsergame #arcadegame</t>
         </is>
       </c>
-      <c r="L11" s="6" t="inlineStr">
+      <c r="L13" s="6" t="inlineStr">
         <is>
           <t>today every pilot flies starfall: the sky opens early. shields are scarce. three attempts. free, in your browser.</t>
         </is>
       </c>
-      <c r="M11" s="6" t="n"/>
-      <c r="N11" s="5" t="inlineStr">
+      <c r="M13" s="6" t="n"/>
+      <c r="N13" s="5" t="inlineStr">
         <is>
           <t>STARFALL DAY: Today's ORION Patrol (Day 50)</t>
         </is>
       </c>
-      <c r="O11" s="6" t="inlineStr">
+      <c r="O13" s="6" t="inlineStr">
         <is>
           <t>Today's shared seed: STARFALL. Meteor rain from the first seconds. Shield is the only drop, and it is late. Every pilot flies the same run. Three attempts, free in your browser.
 Play now: https://surviveorion.com
@@ -1289,70 +1432,70 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="60" customHeight="1">
-      <c r="A12" s="5" t="inlineStr">
+    <row r="14" ht="60" customHeight="1">
+      <c r="A14" s="5" t="inlineStr">
         <is>
           <t>2026-09-02</t>
         </is>
       </c>
-      <c r="B12" s="5" t="inlineStr">
+      <c r="B14" s="5" t="inlineStr">
         <is>
           <t>Wed</t>
         </is>
       </c>
-      <c r="C12" s="5" t="inlineStr">
+      <c r="C14" s="5" t="inlineStr">
         <is>
           <t>TODAY'S PATROL</t>
         </is>
       </c>
-      <c r="D12" s="5" t="inlineStr">
+      <c r="D14" s="5" t="inlineStr">
         <is>
           <t>RED ALERT</t>
         </is>
       </c>
-      <c r="E12" s="6" t="inlineStr">
+      <c r="E14" s="6" t="inlineStr">
         <is>
           <t>Klaxons up. Everything moves faster except you.</t>
         </is>
       </c>
-      <c r="F12" s="5" t="n"/>
-      <c r="G12" s="5" t="inlineStr">
+      <c r="F14" s="5" t="n"/>
+      <c r="G14" s="5" t="inlineStr">
         <is>
           <t>0902_patrol_redalert_916.mov</t>
         </is>
       </c>
-      <c r="H12" s="7" t="inlineStr">
+      <c r="H14" s="7" t="inlineStr">
         <is>
           <t>Not linked yet</t>
         </is>
       </c>
-      <c r="I12" s="5" t="inlineStr">
+      <c r="I14" s="5" t="inlineStr">
         <is>
           <t>Draft</t>
         </is>
       </c>
-      <c r="J12" s="6" t="inlineStr">
+      <c r="J14" s="6" t="inlineStr">
         <is>
           <t>Today every pilot flies RED ALERT: Klaxons up. Everything moves faster except you. Three attempts. Free, in your browser.</t>
         </is>
       </c>
-      <c r="K12" s="5" t="inlineStr">
+      <c r="K14" s="5" t="inlineStr">
         <is>
           <t>#dailychallenge #indiegame #browsergame #arcadegame</t>
         </is>
       </c>
-      <c r="L12" s="6" t="inlineStr">
+      <c r="L14" s="6" t="inlineStr">
         <is>
           <t>today every pilot flies red alert: klaxons up. everything moves faster except you. three attempts. free, in your browser.</t>
         </is>
       </c>
-      <c r="M12" s="6" t="n"/>
-      <c r="N12" s="5" t="inlineStr">
+      <c r="M14" s="6" t="n"/>
+      <c r="N14" s="5" t="inlineStr">
         <is>
           <t>RED ALERT DAY: Today's ORION Patrol (Day 51)</t>
         </is>
       </c>
-      <c r="O12" s="6" t="inlineStr">
+      <c r="O14" s="6" t="inlineStr">
         <is>
           <t>Today's shared seed: RED ALERT. Spawn rate, formation frequency, and pickup drops all sped up. Drone speed is unchanged. Every pilot flies the same run. Three attempts, free in your browser.
 Play now: https://surviveorion.com
@@ -1360,70 +1503,70 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="60" customHeight="1">
-      <c r="A13" s="5" t="inlineStr">
+    <row r="15" ht="60" customHeight="1">
+      <c r="A15" s="5" t="inlineStr">
         <is>
           <t>2026-09-03</t>
         </is>
       </c>
-      <c r="B13" s="5" t="inlineStr">
+      <c r="B15" s="5" t="inlineStr">
         <is>
           <t>Thu</t>
         </is>
       </c>
-      <c r="C13" s="5" t="inlineStr">
+      <c r="C15" s="5" t="inlineStr">
         <is>
           <t>NEW BEST</t>
         </is>
       </c>
-      <c r="D13" s="5" t="inlineStr">
+      <c r="D15" s="5" t="inlineStr">
         <is>
           <t>NEW BEST</t>
         </is>
       </c>
-      <c r="E13" s="6" t="inlineStr">
+      <c r="E15" s="6" t="inlineStr">
         <is>
           <t>Any run that beats your HUD best. The in-app celebration sound is already the hook, cut around it.</t>
         </is>
       </c>
-      <c r="F13" s="5" t="inlineStr"/>
-      <c r="G13" s="5" t="inlineStr">
+      <c r="F15" s="5" t="inlineStr"/>
+      <c r="G15" s="5" t="inlineStr">
         <is>
           <t>0903_newbest_916.mov</t>
         </is>
       </c>
-      <c r="H13" s="7" t="inlineStr">
+      <c r="H15" s="7" t="inlineStr">
         <is>
           <t>Not linked yet</t>
         </is>
       </c>
-      <c r="I13" s="5" t="inlineStr">
+      <c r="I15" s="5" t="inlineStr">
         <is>
           <t>Draft</t>
         </is>
       </c>
-      <c r="J13" s="6" t="inlineStr">
+      <c r="J15" s="6" t="inlineStr">
         <is>
           <t>new personal best 🏆 same run as every other pilot today. free browser game, link in bio</t>
         </is>
       </c>
-      <c r="K13" s="5" t="inlineStr">
+      <c r="K15" s="5" t="inlineStr">
         <is>
           <t>#indiegame #gamingmemes #personalbest #dailychallenge</t>
         </is>
       </c>
-      <c r="L13" s="6" t="inlineStr">
+      <c r="L15" s="6" t="inlineStr">
         <is>
           <t>new best 🏆 free daily dodge game, link in bio</t>
         </is>
       </c>
-      <c r="M13" s="6" t="inlineStr"/>
-      <c r="N13" s="5" t="inlineStr">
+      <c r="M15" s="6" t="inlineStr"/>
+      <c r="N15" s="5" t="inlineStr">
         <is>
           <t>New Personal Best (ORION Daily Patrol)</t>
         </is>
       </c>
-      <c r="O13" s="6" t="inlineStr">
+      <c r="O15" s="6" t="inlineStr">
         <is>
           <t>Same seed as every pilot today. Free dodging game, three attempts a day.
 Play: https://surviveorion.com
@@ -1431,70 +1574,70 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="60" customHeight="1">
-      <c r="A14" s="5" t="inlineStr">
+    <row r="16" ht="60" customHeight="1">
+      <c r="A16" s="5" t="inlineStr">
         <is>
           <t>2026-09-03</t>
         </is>
       </c>
-      <c r="B14" s="5" t="inlineStr">
+      <c r="B16" s="5" t="inlineStr">
         <is>
           <t>Thu</t>
         </is>
       </c>
-      <c r="C14" s="5" t="inlineStr">
+      <c r="C16" s="5" t="inlineStr">
         <is>
           <t>TODAY'S PATROL</t>
         </is>
       </c>
-      <c r="D14" s="5" t="inlineStr">
+      <c r="D16" s="5" t="inlineStr">
         <is>
           <t>THE FLOOD</t>
         </is>
       </c>
-      <c r="E14" s="6" t="inlineStr">
+      <c r="E16" s="6" t="inlineStr">
         <is>
           <t>No formations. They just keep popping in.</t>
         </is>
       </c>
-      <c r="F14" s="5" t="n"/>
-      <c r="G14" s="5" t="inlineStr">
+      <c r="F16" s="5" t="n"/>
+      <c r="G16" s="5" t="inlineStr">
         <is>
           <t>0903_patrol_theflood_916.mov</t>
         </is>
       </c>
-      <c r="H14" s="7" t="inlineStr">
+      <c r="H16" s="7" t="inlineStr">
         <is>
           <t>Not linked yet</t>
         </is>
       </c>
-      <c r="I14" s="5" t="inlineStr">
+      <c r="I16" s="5" t="inlineStr">
         <is>
           <t>Draft</t>
         </is>
       </c>
-      <c r="J14" s="6" t="inlineStr">
+      <c r="J16" s="6" t="inlineStr">
         <is>
           <t>Today every pilot flies THE FLOOD: No formations. They just keep popping in. Three attempts. Free, in your browser.</t>
         </is>
       </c>
-      <c r="K14" s="5" t="inlineStr">
+      <c r="K16" s="5" t="inlineStr">
         <is>
           <t>#dailychallenge #indiegame #browsergame #arcadegame</t>
         </is>
       </c>
-      <c r="L14" s="6" t="inlineStr">
+      <c r="L16" s="6" t="inlineStr">
         <is>
           <t>today every pilot flies the flood: no formations. they just keep popping in. three attempts. free, in your browser.</t>
         </is>
       </c>
-      <c r="M14" s="6" t="n"/>
-      <c r="N14" s="5" t="inlineStr">
+      <c r="M16" s="6" t="n"/>
+      <c r="N16" s="5" t="inlineStr">
         <is>
           <t>THE FLOOD DAY: Today's ORION Patrol (Day 52)</t>
         </is>
       </c>
-      <c r="O14" s="6" t="inlineStr">
+      <c r="O16" s="6" t="inlineStr">
         <is>
           <t>Today's shared seed: THE FLOOD. A constant beat from the edges. The beat speeds up the whole run. Every pilot flies the same run. Three attempts, free in your browser.
 Play now: https://surviveorion.com
@@ -1502,70 +1645,70 @@
         </is>
       </c>
     </row>
-    <row r="15" ht="60" customHeight="1">
-      <c r="A15" s="5" t="inlineStr">
+    <row r="17" ht="60" customHeight="1">
+      <c r="A17" s="5" t="inlineStr">
         <is>
           <t>2026-09-04</t>
         </is>
       </c>
-      <c r="B15" s="5" t="inlineStr">
+      <c r="B17" s="5" t="inlineStr">
         <is>
           <t>Fri</t>
         </is>
       </c>
-      <c r="C15" s="5" t="inlineStr">
+      <c r="C17" s="5" t="inlineStr">
         <is>
           <t>TODAY'S PATROL</t>
         </is>
       </c>
-      <c r="D15" s="5" t="inlineStr">
+      <c r="D17" s="5" t="inlineStr">
         <is>
           <t>THUNDER</t>
         </is>
       </c>
-      <c r="E15" s="6" t="inlineStr">
+      <c r="E17" s="6" t="inlineStr">
         <is>
           <t>Aim the ray. Let it hop.</t>
         </is>
       </c>
-      <c r="F15" s="5" t="n"/>
-      <c r="G15" s="5" t="inlineStr">
+      <c r="F17" s="5" t="n"/>
+      <c r="G17" s="5" t="inlineStr">
         <is>
           <t>0904_patrol_thunder_916.mov</t>
         </is>
       </c>
-      <c r="H15" s="7" t="inlineStr">
+      <c r="H17" s="7" t="inlineStr">
         <is>
           <t>Not linked yet</t>
         </is>
       </c>
-      <c r="I15" s="5" t="inlineStr">
+      <c r="I17" s="5" t="inlineStr">
         <is>
           <t>Draft</t>
         </is>
       </c>
-      <c r="J15" s="6" t="inlineStr">
+      <c r="J17" s="6" t="inlineStr">
         <is>
           <t>Today every pilot flies THUNDER: Aim the ray. Let it hop. Three attempts. Free, in your browser.</t>
         </is>
       </c>
-      <c r="K15" s="5" t="inlineStr">
+      <c r="K17" s="5" t="inlineStr">
         <is>
           <t>#dailychallenge #indiegame #browsergame #arcadegame</t>
         </is>
       </c>
-      <c r="L15" s="6" t="inlineStr">
+      <c r="L17" s="6" t="inlineStr">
         <is>
           <t>today every pilot flies thunder: aim the ray. let it hop. three attempts. free, in your browser.</t>
         </is>
       </c>
-      <c r="M15" s="6" t="n"/>
-      <c r="N15" s="5" t="inlineStr">
+      <c r="M17" s="6" t="n"/>
+      <c r="N17" s="5" t="inlineStr">
         <is>
           <t>THUNDER DAY: Today's ORION Patrol (Day 53)</t>
         </is>
       </c>
-      <c r="O15" s="6" t="inlineStr">
+      <c r="O17" s="6" t="inlineStr">
         <is>
           <t>Today's shared seed: THUNDER. Every pickup is Thunder. A lightning ray along your nose. Each kill sparks Arc hops. Ray kills pay double. Every pilot flies the same run. Three attempts, free in your browser.
 Play now: https://surviveorion.com
@@ -1573,70 +1716,70 @@
         </is>
       </c>
     </row>
-    <row r="16" ht="60" customHeight="1">
-      <c r="A16" s="5" t="inlineStr">
+    <row r="18" ht="60" customHeight="1">
+      <c r="A18" s="5" t="inlineStr">
         <is>
           <t>2026-09-05</t>
         </is>
       </c>
-      <c r="B16" s="5" t="inlineStr">
+      <c r="B18" s="5" t="inlineStr">
         <is>
           <t>Sat</t>
         </is>
       </c>
-      <c r="C16" s="5" t="inlineStr">
+      <c r="C18" s="5" t="inlineStr">
         <is>
           <t>THE BOARD</t>
         </is>
       </c>
-      <c r="D16" s="5" t="inlineStr">
+      <c r="D18" s="5" t="inlineStr">
         <is>
           <t>Beaten by a stranger</t>
         </is>
       </c>
-      <c r="E16" s="6" t="inlineStr">
+      <c r="E18" s="6" t="inlineStr">
         <is>
           <t>Your best run of the day, then the board showing someone above you right now. Ends on the gap, not the score.</t>
         </is>
       </c>
-      <c r="F16" s="5" t="inlineStr"/>
-      <c r="G16" s="5" t="inlineStr">
+      <c r="F18" s="5" t="inlineStr"/>
+      <c r="G18" s="5" t="inlineStr">
         <is>
           <t>0905_beatenbystranger_916.mov</t>
         </is>
       </c>
-      <c r="H16" s="7" t="inlineStr">
+      <c r="H18" s="7" t="inlineStr">
         <is>
           <t>Not linked yet</t>
         </is>
       </c>
-      <c r="I16" s="5" t="inlineStr">
+      <c r="I18" s="5" t="inlineStr">
         <is>
           <t>Draft</t>
         </is>
       </c>
-      <c r="J16" s="6" t="inlineStr">
+      <c r="J18" s="6" t="inlineStr">
         <is>
           <t>my best run today. someone's already ahead of it 😭 same seed, same day, go beat them. link in bio</t>
         </is>
       </c>
-      <c r="K16" s="5" t="inlineStr">
+      <c r="K18" s="5" t="inlineStr">
         <is>
           <t>#dailychallenge #indiegame #gamingmemes #leaderboard</t>
         </is>
       </c>
-      <c r="L16" s="6" t="inlineStr">
+      <c r="L18" s="6" t="inlineStr">
         <is>
           <t>my best today. this guy's best today 💀 same run, same day, link in bio</t>
         </is>
       </c>
-      <c r="M16" s="6" t="inlineStr"/>
-      <c r="N16" s="5" t="inlineStr">
+      <c r="M18" s="6" t="inlineStr"/>
+      <c r="N18" s="5" t="inlineStr">
         <is>
           <t>Someone Already Beat My Best Run Today (ORION)</t>
         </is>
       </c>
-      <c r="O16" s="6" t="inlineStr">
+      <c r="O18" s="6" t="inlineStr">
         <is>
           <t>Same seed as every pilot. The board never sits still. Free dodging game, three attempts a day.
 Play: https://surviveorion.com
@@ -1644,70 +1787,70 @@
         </is>
       </c>
     </row>
-    <row r="17" ht="60" customHeight="1">
-      <c r="A17" s="5" t="inlineStr">
+    <row r="19" ht="60" customHeight="1">
+      <c r="A19" s="5" t="inlineStr">
         <is>
           <t>2026-09-05</t>
         </is>
       </c>
-      <c r="B17" s="5" t="inlineStr">
+      <c r="B19" s="5" t="inlineStr">
         <is>
           <t>Sat</t>
         </is>
       </c>
-      <c r="C17" s="5" t="inlineStr">
+      <c r="C19" s="5" t="inlineStr">
         <is>
           <t>TODAY'S PATROL</t>
         </is>
       </c>
-      <c r="D17" s="5" t="inlineStr">
+      <c r="D19" s="5" t="inlineStr">
         <is>
           <t>YEAR OF THE SERPENT</t>
         </is>
       </c>
-      <c r="E17" s="6" t="inlineStr">
+      <c r="E19" s="6" t="inlineStr">
         <is>
           <t>Every formation slithers today. Watch the trains.</t>
         </is>
       </c>
-      <c r="F17" s="5" t="n"/>
-      <c r="G17" s="5" t="inlineStr">
+      <c r="F19" s="5" t="n"/>
+      <c r="G19" s="5" t="inlineStr">
         <is>
           <t>0905_patrol_yearoftheserpent_916.mov</t>
         </is>
       </c>
-      <c r="H17" s="7" t="inlineStr">
+      <c r="H19" s="7" t="inlineStr">
         <is>
           <t>Not linked yet</t>
         </is>
       </c>
-      <c r="I17" s="5" t="inlineStr">
+      <c r="I19" s="5" t="inlineStr">
         <is>
           <t>Draft</t>
         </is>
       </c>
-      <c r="J17" s="6" t="inlineStr">
+      <c r="J19" s="6" t="inlineStr">
         <is>
           <t>Today every pilot flies YEAR OF THE SERPENT: Every formation slithers today. Watch the trains. Three attempts. Free, in your browser.</t>
         </is>
       </c>
-      <c r="K17" s="5" t="inlineStr">
+      <c r="K19" s="5" t="inlineStr">
         <is>
           <t>#dailychallenge #indiegame #browsergame #arcadegame</t>
         </is>
       </c>
-      <c r="L17" s="6" t="inlineStr">
+      <c r="L19" s="6" t="inlineStr">
         <is>
           <t>today every pilot flies year of the serpent: every formation slithers today. watch the trains. three attempts. free, in your browser.</t>
         </is>
       </c>
-      <c r="M17" s="6" t="n"/>
-      <c r="N17" s="5" t="inlineStr">
+      <c r="M19" s="6" t="n"/>
+      <c r="N19" s="5" t="inlineStr">
         <is>
           <t>YEAR OF THE SERPENT DAY: Today's ORION Patrol (Day 54)</t>
         </is>
       </c>
-      <c r="O17" s="6" t="inlineStr">
+      <c r="O19" s="6" t="inlineStr">
         <is>
           <t>Today's shared seed: YEAR OF THE SERPENT. No ambient drones at all. Only serpent trains, more of them, released to hunt after their sweep. Deep in the run the trains keep coming faster and stray drones start leaking in. Every pilot flies the same run. Three attempts, free in your browser.
 Play now: https://surviveorion.com
@@ -1715,74 +1858,74 @@
         </is>
       </c>
     </row>
-    <row r="18" ht="60" customHeight="1">
-      <c r="A18" s="5" t="inlineStr">
+    <row r="20" ht="60" customHeight="1">
+      <c r="A20" s="5" t="inlineStr">
         <is>
           <t>2026-09-06</t>
         </is>
       </c>
-      <c r="B18" s="5" t="inlineStr">
+      <c r="B20" s="5" t="inlineStr">
         <is>
           <t>Sun</t>
         </is>
       </c>
-      <c r="C18" s="5" t="inlineStr">
+      <c r="C20" s="5" t="inlineStr">
         <is>
           <t>TODAY'S PATROL · SUNDAY DOUBLE</t>
         </is>
       </c>
-      <c r="D18" s="5" t="inlineStr">
+      <c r="D20" s="5" t="inlineStr">
         <is>
           <t>PATROL: MAGNETIC FIELD + CLOAK</t>
         </is>
       </c>
-      <c r="E18" s="6" t="inlineStr">
+      <c r="E20" s="6" t="inlineStr">
         <is>
           <t>The pickups want to find you today. They lose the lock. You seed the dark.</t>
         </is>
       </c>
-      <c r="F18" s="5" t="inlineStr">
+      <c r="F20" s="5" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="G18" s="5" t="inlineStr">
+      <c r="G20" s="5" t="inlineStr">
         <is>
           <t>0906_patrol_magneticfieldcloak_916.mov</t>
         </is>
       </c>
-      <c r="H18" s="7" t="inlineStr">
+      <c r="H20" s="7" t="inlineStr">
         <is>
           <t>Not linked yet</t>
         </is>
       </c>
-      <c r="I18" s="5" t="inlineStr">
+      <c r="I20" s="5" t="inlineStr">
         <is>
           <t>Draft</t>
         </is>
       </c>
-      <c r="J18" s="6" t="inlineStr">
+      <c r="J20" s="6" t="inlineStr">
         <is>
           <t>Today every pilot flies MAGNETIC FIELD + CLOAK: The pickups want to find you today. They lose the lock. You seed the dark. Three attempts. Free, in your browser.</t>
         </is>
       </c>
-      <c r="K18" s="5" t="inlineStr">
+      <c r="K20" s="5" t="inlineStr">
         <is>
           <t>#dailychallenge #indiegame #browsergame #arcadegame</t>
         </is>
       </c>
-      <c r="L18" s="6" t="inlineStr">
+      <c r="L20" s="6" t="inlineStr">
         <is>
           <t>today every pilot flies magnetic field + cloak: the pickups want to find you today. they lose the lock. you seed the dark. three attempts. free, in your browser.</t>
         </is>
       </c>
-      <c r="M18" s="6" t="n"/>
-      <c r="N18" s="5" t="inlineStr">
+      <c r="M20" s="6" t="n"/>
+      <c r="N20" s="5" t="inlineStr">
         <is>
           <t>MAGNETIC FIELD + CLOAK DAY: Today's ORION Patrol (Day 55)</t>
         </is>
       </c>
-      <c r="O18" s="6" t="inlineStr">
+      <c r="O20" s="6" t="inlineStr">
         <is>
           <t>Today's shared seed: MAGNETIC FIELD + CLOAK. Pickups slowly drift toward your ship all day, on top of their normal wander. Every pickup is Cloak. Drones hover, lost. Invisible bombs drop along your path and explode when you reappear. Every pilot flies the same run. Three attempts, free in your browser.
 Play now: https://surviveorion.com
@@ -1790,70 +1933,70 @@
         </is>
       </c>
     </row>
-    <row r="19" ht="60" customHeight="1">
-      <c r="A19" s="5" t="inlineStr">
+    <row r="21" ht="60" customHeight="1">
+      <c r="A21" s="5" t="inlineStr">
         <is>
           <t>2026-09-07</t>
         </is>
       </c>
-      <c r="B19" s="5" t="inlineStr">
+      <c r="B21" s="5" t="inlineStr">
         <is>
           <t>Mon</t>
         </is>
       </c>
-      <c r="C19" s="5" t="inlineStr">
+      <c r="C21" s="5" t="inlineStr">
         <is>
           <t>BUG</t>
         </is>
       </c>
-      <c r="D19" s="5" t="inlineStr">
+      <c r="D21" s="5" t="inlineStr">
         <is>
           <t>Bug of the week</t>
         </is>
       </c>
-      <c r="E19" s="6" t="inlineStr">
+      <c r="E21" s="6" t="inlineStr">
         <is>
           <t>Any real glitch, physics jank, or weird interaction. Film it as-is, matter-of-fact caption, no apology. "Who needs new features when you got old bugs."</t>
         </is>
       </c>
-      <c r="F19" s="5" t="inlineStr"/>
-      <c r="G19" s="5" t="inlineStr">
+      <c r="F21" s="5" t="inlineStr"/>
+      <c r="G21" s="5" t="inlineStr">
         <is>
           <t>0907_bugoftheweek_916.mov</t>
         </is>
       </c>
-      <c r="H19" s="7" t="inlineStr">
+      <c r="H21" s="7" t="inlineStr">
         <is>
           <t>Not linked yet</t>
         </is>
       </c>
-      <c r="I19" s="5" t="inlineStr">
+      <c r="I21" s="5" t="inlineStr">
         <is>
           <t>Draft</t>
         </is>
       </c>
-      <c r="J19" s="6" t="inlineStr">
+      <c r="J21" s="6" t="inlineStr">
         <is>
           <t>bug of the week. we see it too. free browser game, link in bio</t>
         </is>
       </c>
-      <c r="K19" s="5" t="inlineStr">
+      <c r="K21" s="5" t="inlineStr">
         <is>
           <t>#gamedev #indiegame #gamingmemes #bug</t>
         </is>
       </c>
-      <c r="L19" s="6" t="inlineStr">
+      <c r="L21" s="6" t="inlineStr">
         <is>
           <t>bug of the week 💀 nobody's perfect, free daily dodge game, link in bio</t>
         </is>
       </c>
-      <c r="M19" s="6" t="inlineStr"/>
-      <c r="N19" s="5" t="inlineStr">
+      <c r="M21" s="6" t="inlineStr"/>
+      <c r="N21" s="5" t="inlineStr">
         <is>
           <t>Bug of the Week (ORION Devlog Clip)</t>
         </is>
       </c>
-      <c r="O19" s="6" t="inlineStr">
+      <c r="O21" s="6" t="inlineStr">
         <is>
           <t>Real jank, filmed as it happened. Free daily dodging game.
 Play: https://surviveorion.com
@@ -1861,70 +2004,70 @@
         </is>
       </c>
     </row>
-    <row r="20" ht="60" customHeight="1">
-      <c r="A20" s="5" t="inlineStr">
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
         <is>
           <t>2026-09-07</t>
         </is>
       </c>
-      <c r="B20" s="5" t="inlineStr">
+      <c r="B22" s="5" t="inlineStr">
         <is>
           <t>Mon</t>
         </is>
       </c>
-      <c r="C20" s="5" t="inlineStr">
+      <c r="C22" s="5" t="inlineStr">
         <is>
           <t>TODAY'S PATROL</t>
         </is>
       </c>
-      <c r="D20" s="5" t="inlineStr">
+      <c r="D22" s="5" t="inlineStr">
         <is>
           <t>RAM RAID</t>
         </is>
       </c>
-      <c r="E20" s="6" t="inlineStr">
+      <c r="E22" s="6" t="inlineStr">
         <is>
           <t>The shell is short. Spend it, then dodge naked.</t>
         </is>
       </c>
-      <c r="F20" s="5" t="n"/>
-      <c r="G20" s="5" t="inlineStr">
+      <c r="F22" s="5" t="n"/>
+      <c r="G22" s="5" t="inlineStr">
         <is>
           <t>0907_patrol_ramraid_916.mov</t>
         </is>
       </c>
-      <c r="H20" s="7" t="inlineStr">
+      <c r="H22" s="7" t="inlineStr">
         <is>
           <t>Not linked yet</t>
         </is>
       </c>
-      <c r="I20" s="5" t="inlineStr">
+      <c r="I22" s="5" t="inlineStr">
         <is>
           <t>Draft</t>
         </is>
       </c>
-      <c r="J20" s="6" t="inlineStr">
+      <c r="J22" s="6" t="inlineStr">
         <is>
           <t>Today every pilot flies RAM RAID: The shell is short. Spend it, then dodge naked. Three attempts. Free, in your browser.</t>
         </is>
       </c>
-      <c r="K20" s="5" t="inlineStr">
+      <c r="K22" s="5" t="inlineStr">
         <is>
           <t>#dailychallenge #indiegame #browsergame #arcadegame</t>
         </is>
       </c>
-      <c r="L20" s="6" t="inlineStr">
+      <c r="L22" s="6" t="inlineStr">
         <is>
           <t>today every pilot flies ram raid: the shell is short. spend it, then dodge naked. three attempts. free, in your browser.</t>
         </is>
       </c>
-      <c r="M20" s="6" t="n"/>
-      <c r="N20" s="5" t="inlineStr">
+      <c r="M22" s="6" t="n"/>
+      <c r="N22" s="5" t="inlineStr">
         <is>
           <t>RAM RAID DAY: Today's ORION Patrol (Day 56)</t>
         </is>
       </c>
-      <c r="O20" s="6" t="inlineStr">
+      <c r="O22" s="6" t="inlineStr">
         <is>
           <t>Today's shared seed: RAM RAID. Starshell is the only drop, and it is scarce. The shell lasts about two seconds. You are invincible while it is up. Every pilot flies the same run. Three attempts, free in your browser.
 Play now: https://surviveorion.com
@@ -1932,70 +2075,70 @@
         </is>
       </c>
     </row>
-    <row r="21" ht="60" customHeight="1">
-      <c r="A21" s="5" t="inlineStr">
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
         <is>
           <t>2026-09-08</t>
         </is>
       </c>
-      <c r="B21" s="5" t="inlineStr">
+      <c r="B23" s="5" t="inlineStr">
         <is>
           <t>Tue</t>
         </is>
       </c>
-      <c r="C21" s="5" t="inlineStr">
+      <c r="C23" s="5" t="inlineStr">
         <is>
           <t>TODAY'S PATROL</t>
         </is>
       </c>
-      <c r="D21" s="5" t="inlineStr">
+      <c r="D23" s="5" t="inlineStr">
         <is>
           <t>SINGULARITY</t>
         </is>
       </c>
-      <c r="E21" s="6" t="inlineStr">
+      <c r="E23" s="6" t="inlineStr">
         <is>
           <t>The banned singularity is back for one day. Use it well.</t>
         </is>
       </c>
-      <c r="F21" s="5" t="n"/>
-      <c r="G21" s="5" t="inlineStr">
+      <c r="F23" s="5" t="n"/>
+      <c r="G23" s="5" t="inlineStr">
         <is>
           <t>0908_patrol_singularity_916.mov</t>
         </is>
       </c>
-      <c r="H21" s="7" t="inlineStr">
+      <c r="H23" s="7" t="inlineStr">
         <is>
           <t>Not linked yet</t>
         </is>
       </c>
-      <c r="I21" s="5" t="inlineStr">
+      <c r="I23" s="5" t="inlineStr">
         <is>
           <t>Draft</t>
         </is>
       </c>
-      <c r="J21" s="6" t="inlineStr">
+      <c r="J23" s="6" t="inlineStr">
         <is>
           <t>Today every pilot flies SINGULARITY: The banned singularity is back for one day. Use it well. Three attempts. Free, in your browser.</t>
         </is>
       </c>
-      <c r="K21" s="5" t="inlineStr">
+      <c r="K23" s="5" t="inlineStr">
         <is>
           <t>#dailychallenge #indiegame #browsergame #arcadegame</t>
         </is>
       </c>
-      <c r="L21" s="6" t="inlineStr">
+      <c r="L23" s="6" t="inlineStr">
         <is>
           <t>today every pilot flies singularity: the banned singularity is back for one day. use it well. three attempts. free, in your browser.</t>
         </is>
       </c>
-      <c r="M21" s="6" t="n"/>
-      <c r="N21" s="5" t="inlineStr">
+      <c r="M23" s="6" t="n"/>
+      <c r="N23" s="5" t="inlineStr">
         <is>
           <t>SINGULARITY DAY: Today's ORION Patrol (Day 57)</t>
         </is>
       </c>
-      <c r="O21" s="6" t="inlineStr">
+      <c r="O23" s="6" t="inlineStr">
         <is>
           <t>Today's shared seed: SINGULARITY. Vortex (normally benched) drops often today. Every pilot flies the same run. Three attempts, free in your browser.
 Play now: https://surviveorion.com
@@ -2003,68 +2146,68 @@
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
+    <row r="24">
+      <c r="A24" t="inlineStr">
         <is>
           <t>2026-09-26</t>
         </is>
       </c>
-      <c r="B22" t="inlineStr">
+      <c r="B24" t="inlineStr">
         <is>
           <t>Sat</t>
         </is>
       </c>
-      <c r="C22" t="inlineStr">
+      <c r="C24" t="inlineStr">
         <is>
           <t>TODAY'S PATROL</t>
         </is>
       </c>
-      <c r="D22" t="inlineStr">
+      <c r="D24" t="inlineStr">
         <is>
           <t>GREAT WALL</t>
         </is>
       </c>
-      <c r="E22" t="inlineStr">
+      <c r="E24" t="inlineStr">
         <is>
           <t>nothing but walls today.</t>
         </is>
       </c>
-      <c r="G22" t="inlineStr">
+      <c r="G24" t="inlineStr">
         <is>
           <t>0827_greatwall_916.mov</t>
         </is>
       </c>
-      <c r="H22" t="inlineStr">
+      <c r="H24" t="inlineStr">
         <is>
           <t>Linked</t>
         </is>
       </c>
-      <c r="I22" t="inlineStr">
+      <c r="I24" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
       </c>
-      <c r="J22" t="inlineStr">
+      <c r="J24" t="inlineStr">
         <is>
           <t>Today every pilot flies GREAT WALL: nothing but walls today. Three attempts. Free, in your browser.</t>
         </is>
       </c>
-      <c r="K22" t="inlineStr">
+      <c r="K24" t="inlineStr">
         <is>
           <t>#dailychallenge #indiegame #browsergame #arcadegame</t>
         </is>
       </c>
-      <c r="L22" t="inlineStr">
+      <c r="L24" t="inlineStr">
         <is>
           <t>today every pilot flies great wall: nothing but walls today. three attempts. free, in your browser.</t>
         </is>
       </c>
-      <c r="N22" t="inlineStr">
+      <c r="N24" t="inlineStr">
         <is>
           <t>GREAT WALL DAY: Today's ORION Patrol (Day 75)</t>
         </is>
       </c>
-      <c r="O22" t="inlineStr">
+      <c r="O24" t="inlineStr">
         <is>
           <t>Today's shared seed: GREAT WALL. No ambient drones at all. Only walls, mega walls, and pincers, faster than usual, released to hunt after their sweep. Every pilot flies the same run. Three attempts, free in your browser.
 Play now: https://surviveorion.com

</xml_diff>

<commit_message>
Mark the four Buffer-scheduled calendar rows so they are not re-posted. [skip render]
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/ORION_Publishing_Calendar.xlsx
+++ b/ORION_Publishing_Calendar.xlsx
@@ -974,7 +974,7 @@
       </c>
       <c r="I7" s="5" t="inlineStr">
         <is>
-          <t>Approved</t>
+          <t>Scheduled</t>
         </is>
       </c>
       <c r="J7" s="6" t="inlineStr">
@@ -1045,7 +1045,7 @@
       </c>
       <c r="I8" s="5" t="inlineStr">
         <is>
-          <t>Approved</t>
+          <t>Scheduled</t>
         </is>
       </c>
       <c r="J8" s="6" t="inlineStr">
@@ -1114,7 +1114,7 @@
       </c>
       <c r="I9" s="5" t="inlineStr">
         <is>
-          <t>Approved</t>
+          <t>Scheduled</t>
         </is>
       </c>
       <c r="J9" s="6" t="inlineStr">
@@ -1258,7 +1258,7 @@
       </c>
       <c r="I11" s="5" t="inlineStr">
         <is>
-          <t>Approved</t>
+          <t>Scheduled</t>
         </is>
       </c>
       <c r="J11" s="6" t="inlineStr">

</xml_diff>

<commit_message>
Drop the empty Aug 28 WASTED calendar row. [skip render]
WASTED is the same format as SPACE DUST; the draft had no linked clip.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/ORION_Publishing_Calendar.xlsx
+++ b/ORION_Publishing_Calendar.xlsx
@@ -487,7 +487,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O24"/>
+  <dimension ref="A1:O23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -806,57 +806,412 @@
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>WASTED</t>
+          <t>TODAY'S PATROL</t>
         </is>
       </c>
       <c r="D5" s="5" t="inlineStr">
         <is>
-          <t>WASTED classic</t>
+          <t>THE FLOOD</t>
         </is>
       </c>
       <c r="E5" s="6" t="inlineStr">
         <is>
-          <t>Any dumb death. Open the clip mid-chaos, never at the run's start; the shock is the hook.</t>
+          <t>the swarm never stops.</t>
         </is>
       </c>
       <c r="F5" s="5" t="inlineStr"/>
       <c r="G5" s="5" t="inlineStr">
         <is>
-          <t>0828_wastedclassic_916.mov</t>
+          <t>0827_theflood_916.mov</t>
         </is>
       </c>
       <c r="H5" s="7" t="inlineStr">
         <is>
-          <t>Not linked yet</t>
+          <t>Linked</t>
         </is>
       </c>
       <c r="I5" s="5" t="inlineStr">
         <is>
-          <t>Draft</t>
+          <t>Approved</t>
         </is>
       </c>
       <c r="J5" s="6" t="inlineStr">
         <is>
-          <t>flying too close to the stars 💀 (free daily dodge game, link in bio)</t>
+          <t>Today every pilot flies THE FLOOD: the swarm never stops. Three attempts. Free, in your browser.</t>
         </is>
       </c>
       <c r="K5" s="5" t="inlineStr">
         <is>
-          <t>#gamingmemes #indiegame #fail #arcadegame</t>
+          <t>#dailychallenge #indiegame #browsergame #arcadegame</t>
         </is>
       </c>
       <c r="L5" s="6" t="inlineStr">
         <is>
-          <t>the swarm always collects 💀 free daily dodge game, new run every day, link in bio</t>
+          <t>today every pilot flies the flood: the swarm never stops. three attempts. free, in your browser.</t>
         </is>
       </c>
       <c r="M5" s="6" t="inlineStr"/>
       <c r="N5" s="5" t="inlineStr">
         <is>
-          <t>He Really Thought He Had It (ORION)</t>
+          <t>THE FLOOD DAY: Today's ORION Patrol (Day 46)</t>
         </is>
       </c>
       <c r="O5" s="6" t="inlineStr">
+        <is>
+          <t>Today's shared seed: THE FLOOD. Formations almost never happen. Ambient density is up, but arrives in clearer packs with lanes between them. Every pilot flies the same run. Three attempts, free in your browser.
+Play now: https://surviveorion.com
+#dailychallenge #indiegame #browsergame #arcadegame #Shorts</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="60" customHeight="1">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>Sat</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>CLOSE CALL</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>Rate this dodge</t>
+        </is>
+      </c>
+      <c r="E6" s="6" t="inlineStr">
+        <is>
+          <t>Closest-call freeze on the graze, red circle on the gap. No command phrasing, the tagline is just "rate this dodge." The comments do the rest.</t>
+        </is>
+      </c>
+      <c r="F6" s="5" t="inlineStr"/>
+      <c r="G6" s="5" t="inlineStr">
+        <is>
+          <t>0828_ratemydodge_916.mp4</t>
+        </is>
+      </c>
+      <c r="H6" s="7" t="inlineStr">
+        <is>
+          <t>Linked</t>
+        </is>
+      </c>
+      <c r="I6" s="5" t="inlineStr">
+        <is>
+          <t>Scheduled</t>
+        </is>
+      </c>
+      <c r="J6" s="6" t="inlineStr">
+        <is>
+          <t>rate this dodge /10 🛰️</t>
+        </is>
+      </c>
+      <c r="K6" s="5" t="inlineStr">
+        <is>
+          <t>#closecall #gamingmemes #indiegame #dailychallenge</t>
+        </is>
+      </c>
+      <c r="L6" s="6" t="inlineStr">
+        <is>
+          <t>rate the dodge /10 (free daily game, link in bio)</t>
+        </is>
+      </c>
+      <c r="M6" s="6" t="inlineStr"/>
+      <c r="N6" s="5" t="inlineStr">
+        <is>
+          <t>Rate This Dodge /10 (ORION)</t>
+        </is>
+      </c>
+      <c r="O6" s="6" t="inlineStr">
+        <is>
+          <t>How close was too close? Free daily dodging game, same run for every pilot.
+Play: https://surviveorion.com
+#Shorts</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="60" customHeight="1">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>Sat</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>TODAY'S PATROL</t>
+        </is>
+      </c>
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>GOLD DASH</t>
+        </is>
+      </c>
+      <c r="E7" s="6" t="inlineStr">
+        <is>
+          <t>Stop, point, burn the line.</t>
+        </is>
+      </c>
+      <c r="F7" s="5" t="n"/>
+      <c r="G7" s="5" t="inlineStr">
+        <is>
+          <t>0828_GOLDDASH_916.mp4</t>
+        </is>
+      </c>
+      <c r="H7" s="7" t="inlineStr">
+        <is>
+          <t>Linked</t>
+        </is>
+      </c>
+      <c r="I7" s="5" t="inlineStr">
+        <is>
+          <t>Scheduled</t>
+        </is>
+      </c>
+      <c r="J7" s="6" t="inlineStr">
+        <is>
+          <t>Today every pilot flies GOLD DASH: Stop, point, burn the line. Three attempts. Free, in your browser.</t>
+        </is>
+      </c>
+      <c r="K7" s="5" t="inlineStr">
+        <is>
+          <t>#dailychallenge #indiegame #browsergame #arcadegame</t>
+        </is>
+      </c>
+      <c r="L7" s="6" t="inlineStr">
+        <is>
+          <t>today every pilot flies gold dash: stop, point, burn the line. three attempts. free, in your browser.</t>
+        </is>
+      </c>
+      <c r="M7" s="6" t="n"/>
+      <c r="N7" s="5" t="inlineStr">
+        <is>
+          <t>GOLD DASH DAY: Today's ORION Patrol (Day 47)</t>
+        </is>
+      </c>
+      <c r="O7" s="6" t="inlineStr">
+        <is>
+          <t>Today's shared seed: GOLD DASH. Every pickup is Afterburner. Grab one and you freeze, aim, then dash. You ram while aiming and the corridor burns. Another dash always waits across the field. Every pilot flies the same run. Three attempts, free in your browser.
+Play now: https://surviveorion.com
+#dailychallenge #indiegame #browsergame #arcadegame #Shorts</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="60" customHeight="1">
+      <c r="A8" s="8" t="n">
+        <v>46264</v>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>Sun</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>POV</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>Nature's Call</t>
+        </is>
+      </c>
+      <c r="E8" s="6" t="inlineStr">
+        <is>
+          <t>POV: answering nature's call while trying to survive</t>
+        </is>
+      </c>
+      <c r="F8" s="5" t="n"/>
+      <c r="G8" s="5" t="inlineStr">
+        <is>
+          <t>0828_naturecall_916.mp4</t>
+        </is>
+      </c>
+      <c r="H8" s="7" t="inlineStr">
+        <is>
+          <t>Linked</t>
+        </is>
+      </c>
+      <c r="I8" s="5" t="inlineStr">
+        <is>
+          <t>Scheduled</t>
+        </is>
+      </c>
+      <c r="J8" s="6" t="inlineStr">
+        <is>
+          <t>POV: answering nature's call while trying to survive 💀 4x speed. Three attempts. Free browser game, link in bio.</t>
+        </is>
+      </c>
+      <c r="K8" s="5" t="inlineStr">
+        <is>
+          <t>#gamingmemes #indiegame #fail #dailychallenge #browsergame</t>
+        </is>
+      </c>
+      <c r="L8" s="6" t="inlineStr">
+        <is>
+          <t>pov: answering nature's call while trying to survive 💀 free daily dodge game, 3 attempts, link in bio</t>
+        </is>
+      </c>
+      <c r="M8" s="6" t="n"/>
+      <c r="N8" s="5" t="inlineStr">
+        <is>
+          <t>POV: Answering Nature's Call While Trying to Survive (ORION)</t>
+        </is>
+      </c>
+      <c r="O8" s="6" t="inlineStr">
+        <is>
+          <t>4x speed. Same swarm. Nature called anyway. Free daily dodging game, three attempts a day.
+Play: https://surviveorion.com
+#gamingmemes #indiegame #Shorts</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="60" customHeight="1">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>Sun</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>TODAY'S PATROL · SUNDAY DOUBLE</t>
+        </is>
+      </c>
+      <c r="D9" s="5" t="inlineStr">
+        <is>
+          <t>PATROL: BAIT SHOT + YEAR OF THE SERPENT</t>
+        </is>
+      </c>
+      <c r="E9" s="6" t="inlineStr">
+        <is>
+          <t>Pack them, then punch the blob. Every formation slithers today. Watch the trains.</t>
+        </is>
+      </c>
+      <c r="F9" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G9" s="5" t="inlineStr">
+        <is>
+          <t>0830_patrol_baitshotyearoftheserpent_916.mov</t>
+        </is>
+      </c>
+      <c r="H9" s="7" t="inlineStr">
+        <is>
+          <t>Not linked yet</t>
+        </is>
+      </c>
+      <c r="I9" s="5" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="J9" s="6" t="inlineStr">
+        <is>
+          <t>Today every pilot flies BAIT SHOT + YEAR OF THE SERPENT: Pack them, then punch the blob. Every formation slithers today. Watch the trains. Three attempts. Free, in your browser.</t>
+        </is>
+      </c>
+      <c r="K9" s="5" t="inlineStr">
+        <is>
+          <t>#dailychallenge #indiegame #browsergame #arcadegame</t>
+        </is>
+      </c>
+      <c r="L9" s="6" t="inlineStr">
+        <is>
+          <t>today every pilot flies bait shot + year of the serpent: pack them, then punch the blob. every formation slithers today. watch the trains. three attempts. free, in your browser.</t>
+        </is>
+      </c>
+      <c r="M9" s="6" t="n"/>
+      <c r="N9" s="5" t="inlineStr">
+        <is>
+          <t>BAIT SHOT + YEAR OF THE SERPENT DAY: Today's ORION Patrol (Day 48)</t>
+        </is>
+      </c>
+      <c r="O9" s="6" t="inlineStr">
+        <is>
+          <t>Today's shared seed: BAIT SHOT + YEAR OF THE SERPENT. Only Flares and Pulse Shot drop. The flare does not kill. It gathers a blob. Pulse is the shot. No ambient drones at all. Only serpent trains, more of them, released to hunt after their sweep. Deep in the run the trains keep coming faster and stray drones start leaking in. Every pilot flies the same run. Three attempts, free in your browser.
+Play now: https://surviveorion.com
+#dailychallenge #indiegame #browsergame #arcadegame #Shorts</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="60" customHeight="1">
+      <c r="A10" s="8" t="n">
+        <v>46265</v>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>Mon</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>SPACE DUST</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="inlineStr">
+        <is>
+          <t>Space Dust</t>
+        </is>
+      </c>
+      <c r="E10" s="6" t="inlineStr">
+        <is>
+          <t>speedrun to the afterlife</t>
+        </is>
+      </c>
+      <c r="F10" s="5" t="n"/>
+      <c r="G10" s="5" t="inlineStr">
+        <is>
+          <t>0828_spacedust_916.mp4</t>
+        </is>
+      </c>
+      <c r="H10" s="7" t="inlineStr">
+        <is>
+          <t>Linked</t>
+        </is>
+      </c>
+      <c r="I10" s="5" t="inlineStr">
+        <is>
+          <t>Scheduled</t>
+        </is>
+      </c>
+      <c r="J10" s="6" t="inlineStr">
+        <is>
+          <t>speedrun to the afterlife 💀 The daily patrol remains undefeated. Free browser game, link in bio.</t>
+        </is>
+      </c>
+      <c r="K10" s="5" t="inlineStr">
+        <is>
+          <t>#gamingmemes #indiegame #fail #dailychallenge #browsergame</t>
+        </is>
+      </c>
+      <c r="L10" s="6" t="inlineStr">
+        <is>
+          <t>speedrun to the afterlife 💀 free daily dodge game, 3 attempts, new run every day, link in bio</t>
+        </is>
+      </c>
+      <c r="M10" s="6" t="n"/>
+      <c r="N10" s="5" t="inlineStr">
+        <is>
+          <t>Speedrun to the Afterlife (ORION Space Dust)</t>
+        </is>
+      </c>
+      <c r="O10" s="6" t="inlineStr">
         <is>
           <t>The daily patrol is undefeated. Free dodging game, same run for every pilot.
 Play: https://surviveorion.com
@@ -864,496 +1219,70 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="60" customHeight="1">
-      <c r="A6" s="5" t="inlineStr">
-        <is>
-          <t>2026-08-28</t>
-        </is>
-      </c>
-      <c r="B6" s="5" t="inlineStr">
-        <is>
-          <t>Fri</t>
-        </is>
-      </c>
-      <c r="C6" s="5" t="inlineStr">
+    <row r="11" ht="60" customHeight="1">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>Mon</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
         <is>
           <t>TODAY'S PATROL</t>
         </is>
       </c>
-      <c r="D6" s="5" t="inlineStr">
-        <is>
-          <t>THE FLOOD</t>
-        </is>
-      </c>
-      <c r="E6" s="6" t="inlineStr">
-        <is>
-          <t>the swarm never stops.</t>
-        </is>
-      </c>
-      <c r="F6" s="5" t="inlineStr"/>
-      <c r="G6" s="5" t="inlineStr">
-        <is>
-          <t>0827_theflood_916.mov</t>
-        </is>
-      </c>
-      <c r="H6" s="7" t="inlineStr">
-        <is>
-          <t>Linked</t>
-        </is>
-      </c>
-      <c r="I6" s="5" t="inlineStr">
-        <is>
-          <t>Approved</t>
-        </is>
-      </c>
-      <c r="J6" s="6" t="inlineStr">
-        <is>
-          <t>Today every pilot flies THE FLOOD: the swarm never stops. Three attempts. Free, in your browser.</t>
-        </is>
-      </c>
-      <c r="K6" s="5" t="inlineStr">
-        <is>
-          <t>#dailychallenge #indiegame #browsergame #arcadegame</t>
-        </is>
-      </c>
-      <c r="L6" s="6" t="inlineStr">
-        <is>
-          <t>today every pilot flies the flood: the swarm never stops. three attempts. free, in your browser.</t>
-        </is>
-      </c>
-      <c r="M6" s="6" t="inlineStr"/>
-      <c r="N6" s="5" t="inlineStr">
-        <is>
-          <t>THE FLOOD DAY: Today's ORION Patrol (Day 46)</t>
-        </is>
-      </c>
-      <c r="O6" s="6" t="inlineStr">
-        <is>
-          <t>Today's shared seed: THE FLOOD. Formations almost never happen. Ambient density is up, but arrives in clearer packs with lanes between them. Every pilot flies the same run. Three attempts, free in your browser.
-Play now: https://surviveorion.com
-#dailychallenge #indiegame #browsergame #arcadegame #Shorts</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="60" customHeight="1">
-      <c r="A7" s="5" t="inlineStr">
-        <is>
-          <t>2026-08-29</t>
-        </is>
-      </c>
-      <c r="B7" s="5" t="inlineStr">
-        <is>
-          <t>Sat</t>
-        </is>
-      </c>
-      <c r="C7" s="5" t="inlineStr">
-        <is>
-          <t>CLOSE CALL</t>
-        </is>
-      </c>
-      <c r="D7" s="5" t="inlineStr">
-        <is>
-          <t>Rate this dodge</t>
-        </is>
-      </c>
-      <c r="E7" s="6" t="inlineStr">
-        <is>
-          <t>Closest-call freeze on the graze, red circle on the gap. No command phrasing, the tagline is just "rate this dodge." The comments do the rest.</t>
-        </is>
-      </c>
-      <c r="F7" s="5" t="inlineStr"/>
-      <c r="G7" s="5" t="inlineStr">
-        <is>
-          <t>0828_ratemydodge_916.mp4</t>
-        </is>
-      </c>
-      <c r="H7" s="7" t="inlineStr">
-        <is>
-          <t>Linked</t>
-        </is>
-      </c>
-      <c r="I7" s="5" t="inlineStr">
-        <is>
-          <t>Scheduled</t>
-        </is>
-      </c>
-      <c r="J7" s="6" t="inlineStr">
-        <is>
-          <t>rate this dodge /10 🛰️</t>
-        </is>
-      </c>
-      <c r="K7" s="5" t="inlineStr">
-        <is>
-          <t>#closecall #gamingmemes #indiegame #dailychallenge</t>
-        </is>
-      </c>
-      <c r="L7" s="6" t="inlineStr">
-        <is>
-          <t>rate the dodge /10 (free daily game, link in bio)</t>
-        </is>
-      </c>
-      <c r="M7" s="6" t="inlineStr"/>
-      <c r="N7" s="5" t="inlineStr">
-        <is>
-          <t>Rate This Dodge /10 (ORION)</t>
-        </is>
-      </c>
-      <c r="O7" s="6" t="inlineStr">
-        <is>
-          <t>How close was too close? Free daily dodging game, same run for every pilot.
-Play: https://surviveorion.com
-#Shorts</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="60" customHeight="1">
-      <c r="A8" s="5" t="inlineStr">
-        <is>
-          <t>2026-08-29</t>
-        </is>
-      </c>
-      <c r="B8" s="5" t="inlineStr">
-        <is>
-          <t>Sat</t>
-        </is>
-      </c>
-      <c r="C8" s="5" t="inlineStr">
-        <is>
-          <t>TODAY'S PATROL</t>
-        </is>
-      </c>
-      <c r="D8" s="5" t="inlineStr">
-        <is>
-          <t>GOLD DASH</t>
-        </is>
-      </c>
-      <c r="E8" s="6" t="inlineStr">
-        <is>
-          <t>Stop, point, burn the line.</t>
-        </is>
-      </c>
-      <c r="F8" s="5" t="n"/>
-      <c r="G8" s="5" t="inlineStr">
-        <is>
-          <t>0828_GOLDDASH_916.mp4</t>
-        </is>
-      </c>
-      <c r="H8" s="7" t="inlineStr">
-        <is>
-          <t>Linked</t>
-        </is>
-      </c>
-      <c r="I8" s="5" t="inlineStr">
-        <is>
-          <t>Scheduled</t>
-        </is>
-      </c>
-      <c r="J8" s="6" t="inlineStr">
-        <is>
-          <t>Today every pilot flies GOLD DASH: Stop, point, burn the line. Three attempts. Free, in your browser.</t>
-        </is>
-      </c>
-      <c r="K8" s="5" t="inlineStr">
-        <is>
-          <t>#dailychallenge #indiegame #browsergame #arcadegame</t>
-        </is>
-      </c>
-      <c r="L8" s="6" t="inlineStr">
-        <is>
-          <t>today every pilot flies gold dash: stop, point, burn the line. three attempts. free, in your browser.</t>
-        </is>
-      </c>
-      <c r="M8" s="6" t="n"/>
-      <c r="N8" s="5" t="inlineStr">
-        <is>
-          <t>GOLD DASH DAY: Today's ORION Patrol (Day 47)</t>
-        </is>
-      </c>
-      <c r="O8" s="6" t="inlineStr">
-        <is>
-          <t>Today's shared seed: GOLD DASH. Every pickup is Afterburner. Grab one and you freeze, aim, then dash. You ram while aiming and the corridor burns. Another dash always waits across the field. Every pilot flies the same run. Three attempts, free in your browser.
-Play now: https://surviveorion.com
-#dailychallenge #indiegame #browsergame #arcadegame #Shorts</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="60" customHeight="1">
-      <c r="A9" s="8" t="n">
-        <v>46264</v>
-      </c>
-      <c r="B9" s="5" t="inlineStr">
-        <is>
-          <t>Sun</t>
-        </is>
-      </c>
-      <c r="C9" s="5" t="inlineStr">
-        <is>
-          <t>POV</t>
-        </is>
-      </c>
-      <c r="D9" s="5" t="inlineStr">
-        <is>
-          <t>Nature's Call</t>
-        </is>
-      </c>
-      <c r="E9" s="6" t="inlineStr">
-        <is>
-          <t>POV: answering nature's call while trying to survive</t>
-        </is>
-      </c>
-      <c r="F9" s="5" t="n"/>
-      <c r="G9" s="5" t="inlineStr">
-        <is>
-          <t>0828_naturecall_916.mp4</t>
-        </is>
-      </c>
-      <c r="H9" s="7" t="inlineStr">
-        <is>
-          <t>Linked</t>
-        </is>
-      </c>
-      <c r="I9" s="5" t="inlineStr">
-        <is>
-          <t>Scheduled</t>
-        </is>
-      </c>
-      <c r="J9" s="6" t="inlineStr">
-        <is>
-          <t>POV: answering nature's call while trying to survive 💀 4x speed. Three attempts. Free browser game, link in bio.</t>
-        </is>
-      </c>
-      <c r="K9" s="5" t="inlineStr">
-        <is>
-          <t>#gamingmemes #indiegame #fail #dailychallenge #browsergame</t>
-        </is>
-      </c>
-      <c r="L9" s="6" t="inlineStr">
-        <is>
-          <t>pov: answering nature's call while trying to survive 💀 free daily dodge game, 3 attempts, link in bio</t>
-        </is>
-      </c>
-      <c r="M9" s="6" t="n"/>
-      <c r="N9" s="5" t="inlineStr">
-        <is>
-          <t>POV: Answering Nature's Call While Trying to Survive (ORION)</t>
-        </is>
-      </c>
-      <c r="O9" s="6" t="inlineStr">
-        <is>
-          <t>4x speed. Same swarm. Nature called anyway. Free daily dodging game, three attempts a day.
-Play: https://surviveorion.com
-#gamingmemes #indiegame #Shorts</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="60" customHeight="1">
-      <c r="A10" s="5" t="inlineStr">
-        <is>
-          <t>2026-08-30</t>
-        </is>
-      </c>
-      <c r="B10" s="5" t="inlineStr">
-        <is>
-          <t>Sun</t>
-        </is>
-      </c>
-      <c r="C10" s="5" t="inlineStr">
-        <is>
-          <t>TODAY'S PATROL · SUNDAY DOUBLE</t>
-        </is>
-      </c>
-      <c r="D10" s="5" t="inlineStr">
-        <is>
-          <t>PATROL: BAIT SHOT + YEAR OF THE SERPENT</t>
-        </is>
-      </c>
-      <c r="E10" s="6" t="inlineStr">
-        <is>
-          <t>Pack them, then punch the blob. Every formation slithers today. Watch the trains.</t>
-        </is>
-      </c>
-      <c r="F10" s="5" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="G10" s="5" t="inlineStr">
-        <is>
-          <t>0830_patrol_baitshotyearoftheserpent_916.mov</t>
-        </is>
-      </c>
-      <c r="H10" s="7" t="inlineStr">
-        <is>
-          <t>Not linked yet</t>
-        </is>
-      </c>
-      <c r="I10" s="5" t="inlineStr">
-        <is>
-          <t>Draft</t>
-        </is>
-      </c>
-      <c r="J10" s="6" t="inlineStr">
-        <is>
-          <t>Today every pilot flies BAIT SHOT + YEAR OF THE SERPENT: Pack them, then punch the blob. Every formation slithers today. Watch the trains. Three attempts. Free, in your browser.</t>
-        </is>
-      </c>
-      <c r="K10" s="5" t="inlineStr">
-        <is>
-          <t>#dailychallenge #indiegame #browsergame #arcadegame</t>
-        </is>
-      </c>
-      <c r="L10" s="6" t="inlineStr">
-        <is>
-          <t>today every pilot flies bait shot + year of the serpent: pack them, then punch the blob. every formation slithers today. watch the trains. three attempts. free, in your browser.</t>
-        </is>
-      </c>
-      <c r="M10" s="6" t="n"/>
-      <c r="N10" s="5" t="inlineStr">
-        <is>
-          <t>BAIT SHOT + YEAR OF THE SERPENT DAY: Today's ORION Patrol (Day 48)</t>
-        </is>
-      </c>
-      <c r="O10" s="6" t="inlineStr">
-        <is>
-          <t>Today's shared seed: BAIT SHOT + YEAR OF THE SERPENT. Only Flares and Pulse Shot drop. The flare does not kill. It gathers a blob. Pulse is the shot. No ambient drones at all. Only serpent trains, more of them, released to hunt after their sweep. Deep in the run the trains keep coming faster and stray drones start leaking in. Every pilot flies the same run. Three attempts, free in your browser.
-Play now: https://surviveorion.com
-#dailychallenge #indiegame #browsergame #arcadegame #Shorts</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="60" customHeight="1">
-      <c r="A11" s="8" t="n">
-        <v>46265</v>
-      </c>
-      <c r="B11" s="5" t="inlineStr">
-        <is>
-          <t>Mon</t>
-        </is>
-      </c>
-      <c r="C11" s="5" t="inlineStr">
-        <is>
-          <t>SPACE DUST</t>
-        </is>
-      </c>
       <c r="D11" s="5" t="inlineStr">
         <is>
-          <t>Space Dust</t>
+          <t>ION</t>
         </is>
       </c>
       <c r="E11" s="6" t="inlineStr">
         <is>
-          <t>speedrun to the afterlife</t>
+          <t>Shove the line. Let them break each other.</t>
         </is>
       </c>
       <c r="F11" s="5" t="n"/>
       <c r="G11" s="5" t="inlineStr">
         <is>
-          <t>0828_spacedust_916.mp4</t>
+          <t>0831_patrol_ion_916.mov</t>
         </is>
       </c>
       <c r="H11" s="7" t="inlineStr">
         <is>
-          <t>Linked</t>
+          <t>Not linked yet</t>
         </is>
       </c>
       <c r="I11" s="5" t="inlineStr">
         <is>
-          <t>Scheduled</t>
+          <t>Draft</t>
         </is>
       </c>
       <c r="J11" s="6" t="inlineStr">
         <is>
-          <t>speedrun to the afterlife 💀 The daily patrol remains undefeated. Free browser game, link in bio.</t>
+          <t>Today every pilot flies ION: Shove the line. Let them break each other. Three attempts. Free, in your browser.</t>
         </is>
       </c>
       <c r="K11" s="5" t="inlineStr">
         <is>
-          <t>#gamingmemes #indiegame #fail #dailychallenge #browsergame</t>
+          <t>#dailychallenge #indiegame #browsergame #arcadegame</t>
         </is>
       </c>
       <c r="L11" s="6" t="inlineStr">
         <is>
-          <t>speedrun to the afterlife 💀 free daily dodge game, 3 attempts, new run every day, link in bio</t>
+          <t>today every pilot flies ion: shove the line. let them break each other. three attempts. free, in your browser.</t>
         </is>
       </c>
       <c r="M11" s="6" t="n"/>
       <c r="N11" s="5" t="inlineStr">
         <is>
-          <t>Speedrun to the Afterlife (ORION Space Dust)</t>
+          <t>ION DAY: Today's ORION Patrol (Day 49)</t>
         </is>
       </c>
       <c r="O11" s="6" t="inlineStr">
-        <is>
-          <t>The daily patrol is undefeated. Free dodging game, same run for every pilot.
-Play: https://surviveorion.com
-#Shorts</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="60" customHeight="1">
-      <c r="A12" s="5" t="inlineStr">
-        <is>
-          <t>2026-08-31</t>
-        </is>
-      </c>
-      <c r="B12" s="5" t="inlineStr">
-        <is>
-          <t>Mon</t>
-        </is>
-      </c>
-      <c r="C12" s="5" t="inlineStr">
-        <is>
-          <t>TODAY'S PATROL</t>
-        </is>
-      </c>
-      <c r="D12" s="5" t="inlineStr">
-        <is>
-          <t>ION</t>
-        </is>
-      </c>
-      <c r="E12" s="6" t="inlineStr">
-        <is>
-          <t>Shove the line. Let them break each other.</t>
-        </is>
-      </c>
-      <c r="F12" s="5" t="n"/>
-      <c r="G12" s="5" t="inlineStr">
-        <is>
-          <t>0831_patrol_ion_916.mov</t>
-        </is>
-      </c>
-      <c r="H12" s="7" t="inlineStr">
-        <is>
-          <t>Not linked yet</t>
-        </is>
-      </c>
-      <c r="I12" s="5" t="inlineStr">
-        <is>
-          <t>Draft</t>
-        </is>
-      </c>
-      <c r="J12" s="6" t="inlineStr">
-        <is>
-          <t>Today every pilot flies ION: Shove the line. Let them break each other. Three attempts. Free, in your browser.</t>
-        </is>
-      </c>
-      <c r="K12" s="5" t="inlineStr">
-        <is>
-          <t>#dailychallenge #indiegame #browsergame #arcadegame</t>
-        </is>
-      </c>
-      <c r="L12" s="6" t="inlineStr">
-        <is>
-          <t>today every pilot flies ion: shove the line. let them break each other. three attempts. free, in your browser.</t>
-        </is>
-      </c>
-      <c r="M12" s="6" t="n"/>
-      <c r="N12" s="5" t="inlineStr">
-        <is>
-          <t>ION DAY: Today's ORION Patrol (Day 49)</t>
-        </is>
-      </c>
-      <c r="O12" s="6" t="inlineStr">
         <is>
           <t>Today's shared seed: ION. Every pickup is Ion. A forward shockwave pushes drones. The pushed ones live. What they slam dies. Every pilot flies the same run. Three attempts, free in your browser.
 Play now: https://surviveorion.com
@@ -1361,70 +1290,70 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="60" customHeight="1">
-      <c r="A13" s="5" t="inlineStr">
+    <row r="12" ht="60" customHeight="1">
+      <c r="A12" s="5" t="inlineStr">
         <is>
           <t>2026-09-01</t>
         </is>
       </c>
-      <c r="B13" s="5" t="inlineStr">
+      <c r="B12" s="5" t="inlineStr">
         <is>
           <t>Tue</t>
         </is>
       </c>
-      <c r="C13" s="5" t="inlineStr">
+      <c r="C12" s="5" t="inlineStr">
         <is>
           <t>TODAY'S PATROL</t>
         </is>
       </c>
-      <c r="D13" s="5" t="inlineStr">
+      <c r="D12" s="5" t="inlineStr">
         <is>
           <t>STARFALL</t>
         </is>
       </c>
-      <c r="E13" s="6" t="inlineStr">
+      <c r="E12" s="6" t="inlineStr">
         <is>
           <t>The sky opens early. Shields are scarce.</t>
         </is>
       </c>
-      <c r="F13" s="5" t="n"/>
-      <c r="G13" s="5" t="inlineStr">
+      <c r="F12" s="5" t="n"/>
+      <c r="G12" s="5" t="inlineStr">
         <is>
           <t>0901_patrol_starfall_916.mov</t>
         </is>
       </c>
-      <c r="H13" s="7" t="inlineStr">
+      <c r="H12" s="7" t="inlineStr">
         <is>
           <t>Not linked yet</t>
         </is>
       </c>
-      <c r="I13" s="5" t="inlineStr">
+      <c r="I12" s="5" t="inlineStr">
         <is>
           <t>Draft</t>
         </is>
       </c>
-      <c r="J13" s="6" t="inlineStr">
+      <c r="J12" s="6" t="inlineStr">
         <is>
           <t>Today every pilot flies STARFALL: The sky opens early. Shields are scarce. Three attempts. Free, in your browser.</t>
         </is>
       </c>
-      <c r="K13" s="5" t="inlineStr">
+      <c r="K12" s="5" t="inlineStr">
         <is>
           <t>#dailychallenge #indiegame #browsergame #arcadegame</t>
         </is>
       </c>
-      <c r="L13" s="6" t="inlineStr">
+      <c r="L12" s="6" t="inlineStr">
         <is>
           <t>today every pilot flies starfall: the sky opens early. shields are scarce. three attempts. free, in your browser.</t>
         </is>
       </c>
-      <c r="M13" s="6" t="n"/>
-      <c r="N13" s="5" t="inlineStr">
+      <c r="M12" s="6" t="n"/>
+      <c r="N12" s="5" t="inlineStr">
         <is>
           <t>STARFALL DAY: Today's ORION Patrol (Day 50)</t>
         </is>
       </c>
-      <c r="O13" s="6" t="inlineStr">
+      <c r="O12" s="6" t="inlineStr">
         <is>
           <t>Today's shared seed: STARFALL. Meteor rain from the first seconds. Shield is the only drop, and it is late. Every pilot flies the same run. Three attempts, free in your browser.
 Play now: https://surviveorion.com
@@ -1432,70 +1361,70 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="60" customHeight="1">
-      <c r="A14" s="5" t="inlineStr">
+    <row r="13" ht="60" customHeight="1">
+      <c r="A13" s="5" t="inlineStr">
         <is>
           <t>2026-09-02</t>
         </is>
       </c>
-      <c r="B14" s="5" t="inlineStr">
+      <c r="B13" s="5" t="inlineStr">
         <is>
           <t>Wed</t>
         </is>
       </c>
-      <c r="C14" s="5" t="inlineStr">
+      <c r="C13" s="5" t="inlineStr">
         <is>
           <t>TODAY'S PATROL</t>
         </is>
       </c>
-      <c r="D14" s="5" t="inlineStr">
+      <c r="D13" s="5" t="inlineStr">
         <is>
           <t>RED ALERT</t>
         </is>
       </c>
-      <c r="E14" s="6" t="inlineStr">
+      <c r="E13" s="6" t="inlineStr">
         <is>
           <t>Klaxons up. Everything moves faster except you.</t>
         </is>
       </c>
-      <c r="F14" s="5" t="n"/>
-      <c r="G14" s="5" t="inlineStr">
+      <c r="F13" s="5" t="n"/>
+      <c r="G13" s="5" t="inlineStr">
         <is>
           <t>0902_patrol_redalert_916.mov</t>
         </is>
       </c>
-      <c r="H14" s="7" t="inlineStr">
+      <c r="H13" s="7" t="inlineStr">
         <is>
           <t>Not linked yet</t>
         </is>
       </c>
-      <c r="I14" s="5" t="inlineStr">
+      <c r="I13" s="5" t="inlineStr">
         <is>
           <t>Draft</t>
         </is>
       </c>
-      <c r="J14" s="6" t="inlineStr">
+      <c r="J13" s="6" t="inlineStr">
         <is>
           <t>Today every pilot flies RED ALERT: Klaxons up. Everything moves faster except you. Three attempts. Free, in your browser.</t>
         </is>
       </c>
-      <c r="K14" s="5" t="inlineStr">
+      <c r="K13" s="5" t="inlineStr">
         <is>
           <t>#dailychallenge #indiegame #browsergame #arcadegame</t>
         </is>
       </c>
-      <c r="L14" s="6" t="inlineStr">
+      <c r="L13" s="6" t="inlineStr">
         <is>
           <t>today every pilot flies red alert: klaxons up. everything moves faster except you. three attempts. free, in your browser.</t>
         </is>
       </c>
-      <c r="M14" s="6" t="n"/>
-      <c r="N14" s="5" t="inlineStr">
+      <c r="M13" s="6" t="n"/>
+      <c r="N13" s="5" t="inlineStr">
         <is>
           <t>RED ALERT DAY: Today's ORION Patrol (Day 51)</t>
         </is>
       </c>
-      <c r="O14" s="6" t="inlineStr">
+      <c r="O13" s="6" t="inlineStr">
         <is>
           <t>Today's shared seed: RED ALERT. Spawn rate, formation frequency, and pickup drops all sped up. Drone speed is unchanged. Every pilot flies the same run. Three attempts, free in your browser.
 Play now: https://surviveorion.com
@@ -1503,70 +1432,70 @@
         </is>
       </c>
     </row>
-    <row r="15" ht="60" customHeight="1">
-      <c r="A15" s="5" t="inlineStr">
+    <row r="14" ht="60" customHeight="1">
+      <c r="A14" s="5" t="inlineStr">
         <is>
           <t>2026-09-03</t>
         </is>
       </c>
-      <c r="B15" s="5" t="inlineStr">
+      <c r="B14" s="5" t="inlineStr">
         <is>
           <t>Thu</t>
         </is>
       </c>
-      <c r="C15" s="5" t="inlineStr">
+      <c r="C14" s="5" t="inlineStr">
         <is>
           <t>NEW BEST</t>
         </is>
       </c>
-      <c r="D15" s="5" t="inlineStr">
+      <c r="D14" s="5" t="inlineStr">
         <is>
           <t>NEW BEST</t>
         </is>
       </c>
-      <c r="E15" s="6" t="inlineStr">
+      <c r="E14" s="6" t="inlineStr">
         <is>
           <t>Any run that beats your HUD best. The in-app celebration sound is already the hook, cut around it.</t>
         </is>
       </c>
-      <c r="F15" s="5" t="inlineStr"/>
-      <c r="G15" s="5" t="inlineStr">
+      <c r="F14" s="5" t="inlineStr"/>
+      <c r="G14" s="5" t="inlineStr">
         <is>
           <t>0903_newbest_916.mov</t>
         </is>
       </c>
-      <c r="H15" s="7" t="inlineStr">
+      <c r="H14" s="7" t="inlineStr">
         <is>
           <t>Not linked yet</t>
         </is>
       </c>
-      <c r="I15" s="5" t="inlineStr">
+      <c r="I14" s="5" t="inlineStr">
         <is>
           <t>Draft</t>
         </is>
       </c>
-      <c r="J15" s="6" t="inlineStr">
+      <c r="J14" s="6" t="inlineStr">
         <is>
           <t>new personal best 🏆 same run as every other pilot today. free browser game, link in bio</t>
         </is>
       </c>
-      <c r="K15" s="5" t="inlineStr">
+      <c r="K14" s="5" t="inlineStr">
         <is>
           <t>#indiegame #gamingmemes #personalbest #dailychallenge</t>
         </is>
       </c>
-      <c r="L15" s="6" t="inlineStr">
+      <c r="L14" s="6" t="inlineStr">
         <is>
           <t>new best 🏆 free daily dodge game, link in bio</t>
         </is>
       </c>
-      <c r="M15" s="6" t="inlineStr"/>
-      <c r="N15" s="5" t="inlineStr">
+      <c r="M14" s="6" t="inlineStr"/>
+      <c r="N14" s="5" t="inlineStr">
         <is>
           <t>New Personal Best (ORION Daily Patrol)</t>
         </is>
       </c>
-      <c r="O15" s="6" t="inlineStr">
+      <c r="O14" s="6" t="inlineStr">
         <is>
           <t>Same seed as every pilot today. Free dodging game, three attempts a day.
 Play: https://surviveorion.com
@@ -1574,70 +1503,70 @@
         </is>
       </c>
     </row>
-    <row r="16" ht="60" customHeight="1">
-      <c r="A16" s="5" t="inlineStr">
+    <row r="15" ht="60" customHeight="1">
+      <c r="A15" s="5" t="inlineStr">
         <is>
           <t>2026-09-03</t>
         </is>
       </c>
-      <c r="B16" s="5" t="inlineStr">
+      <c r="B15" s="5" t="inlineStr">
         <is>
           <t>Thu</t>
         </is>
       </c>
-      <c r="C16" s="5" t="inlineStr">
+      <c r="C15" s="5" t="inlineStr">
         <is>
           <t>TODAY'S PATROL</t>
         </is>
       </c>
-      <c r="D16" s="5" t="inlineStr">
+      <c r="D15" s="5" t="inlineStr">
         <is>
           <t>THE FLOOD</t>
         </is>
       </c>
-      <c r="E16" s="6" t="inlineStr">
+      <c r="E15" s="6" t="inlineStr">
         <is>
           <t>No formations. They just keep popping in.</t>
         </is>
       </c>
-      <c r="F16" s="5" t="n"/>
-      <c r="G16" s="5" t="inlineStr">
+      <c r="F15" s="5" t="n"/>
+      <c r="G15" s="5" t="inlineStr">
         <is>
           <t>0903_patrol_theflood_916.mov</t>
         </is>
       </c>
-      <c r="H16" s="7" t="inlineStr">
+      <c r="H15" s="7" t="inlineStr">
         <is>
           <t>Not linked yet</t>
         </is>
       </c>
-      <c r="I16" s="5" t="inlineStr">
+      <c r="I15" s="5" t="inlineStr">
         <is>
           <t>Draft</t>
         </is>
       </c>
-      <c r="J16" s="6" t="inlineStr">
+      <c r="J15" s="6" t="inlineStr">
         <is>
           <t>Today every pilot flies THE FLOOD: No formations. They just keep popping in. Three attempts. Free, in your browser.</t>
         </is>
       </c>
-      <c r="K16" s="5" t="inlineStr">
+      <c r="K15" s="5" t="inlineStr">
         <is>
           <t>#dailychallenge #indiegame #browsergame #arcadegame</t>
         </is>
       </c>
-      <c r="L16" s="6" t="inlineStr">
+      <c r="L15" s="6" t="inlineStr">
         <is>
           <t>today every pilot flies the flood: no formations. they just keep popping in. three attempts. free, in your browser.</t>
         </is>
       </c>
-      <c r="M16" s="6" t="n"/>
-      <c r="N16" s="5" t="inlineStr">
+      <c r="M15" s="6" t="n"/>
+      <c r="N15" s="5" t="inlineStr">
         <is>
           <t>THE FLOOD DAY: Today's ORION Patrol (Day 52)</t>
         </is>
       </c>
-      <c r="O16" s="6" t="inlineStr">
+      <c r="O15" s="6" t="inlineStr">
         <is>
           <t>Today's shared seed: THE FLOOD. A constant beat from the edges. The beat speeds up the whole run. Every pilot flies the same run. Three attempts, free in your browser.
 Play now: https://surviveorion.com
@@ -1645,70 +1574,70 @@
         </is>
       </c>
     </row>
-    <row r="17" ht="60" customHeight="1">
-      <c r="A17" s="5" t="inlineStr">
+    <row r="16" ht="60" customHeight="1">
+      <c r="A16" s="5" t="inlineStr">
         <is>
           <t>2026-09-04</t>
         </is>
       </c>
-      <c r="B17" s="5" t="inlineStr">
+      <c r="B16" s="5" t="inlineStr">
         <is>
           <t>Fri</t>
         </is>
       </c>
-      <c r="C17" s="5" t="inlineStr">
+      <c r="C16" s="5" t="inlineStr">
         <is>
           <t>TODAY'S PATROL</t>
         </is>
       </c>
-      <c r="D17" s="5" t="inlineStr">
+      <c r="D16" s="5" t="inlineStr">
         <is>
           <t>THUNDER</t>
         </is>
       </c>
-      <c r="E17" s="6" t="inlineStr">
+      <c r="E16" s="6" t="inlineStr">
         <is>
           <t>Aim the ray. Let it hop.</t>
         </is>
       </c>
-      <c r="F17" s="5" t="n"/>
-      <c r="G17" s="5" t="inlineStr">
+      <c r="F16" s="5" t="n"/>
+      <c r="G16" s="5" t="inlineStr">
         <is>
           <t>0904_patrol_thunder_916.mov</t>
         </is>
       </c>
-      <c r="H17" s="7" t="inlineStr">
+      <c r="H16" s="7" t="inlineStr">
         <is>
           <t>Not linked yet</t>
         </is>
       </c>
-      <c r="I17" s="5" t="inlineStr">
+      <c r="I16" s="5" t="inlineStr">
         <is>
           <t>Draft</t>
         </is>
       </c>
-      <c r="J17" s="6" t="inlineStr">
+      <c r="J16" s="6" t="inlineStr">
         <is>
           <t>Today every pilot flies THUNDER: Aim the ray. Let it hop. Three attempts. Free, in your browser.</t>
         </is>
       </c>
-      <c r="K17" s="5" t="inlineStr">
+      <c r="K16" s="5" t="inlineStr">
         <is>
           <t>#dailychallenge #indiegame #browsergame #arcadegame</t>
         </is>
       </c>
-      <c r="L17" s="6" t="inlineStr">
+      <c r="L16" s="6" t="inlineStr">
         <is>
           <t>today every pilot flies thunder: aim the ray. let it hop. three attempts. free, in your browser.</t>
         </is>
       </c>
-      <c r="M17" s="6" t="n"/>
-      <c r="N17" s="5" t="inlineStr">
+      <c r="M16" s="6" t="n"/>
+      <c r="N16" s="5" t="inlineStr">
         <is>
           <t>THUNDER DAY: Today's ORION Patrol (Day 53)</t>
         </is>
       </c>
-      <c r="O17" s="6" t="inlineStr">
+      <c r="O16" s="6" t="inlineStr">
         <is>
           <t>Today's shared seed: THUNDER. Every pickup is Thunder. A lightning ray along your nose. Each kill sparks Arc hops. Ray kills pay double. Every pilot flies the same run. Three attempts, free in your browser.
 Play now: https://surviveorion.com
@@ -1716,70 +1645,70 @@
         </is>
       </c>
     </row>
-    <row r="18" ht="60" customHeight="1">
-      <c r="A18" s="5" t="inlineStr">
+    <row r="17" ht="60" customHeight="1">
+      <c r="A17" s="5" t="inlineStr">
         <is>
           <t>2026-09-05</t>
         </is>
       </c>
-      <c r="B18" s="5" t="inlineStr">
+      <c r="B17" s="5" t="inlineStr">
         <is>
           <t>Sat</t>
         </is>
       </c>
-      <c r="C18" s="5" t="inlineStr">
+      <c r="C17" s="5" t="inlineStr">
         <is>
           <t>THE BOARD</t>
         </is>
       </c>
-      <c r="D18" s="5" t="inlineStr">
+      <c r="D17" s="5" t="inlineStr">
         <is>
           <t>Beaten by a stranger</t>
         </is>
       </c>
-      <c r="E18" s="6" t="inlineStr">
+      <c r="E17" s="6" t="inlineStr">
         <is>
           <t>Your best run of the day, then the board showing someone above you right now. Ends on the gap, not the score.</t>
         </is>
       </c>
-      <c r="F18" s="5" t="inlineStr"/>
-      <c r="G18" s="5" t="inlineStr">
+      <c r="F17" s="5" t="inlineStr"/>
+      <c r="G17" s="5" t="inlineStr">
         <is>
           <t>0905_beatenbystranger_916.mov</t>
         </is>
       </c>
-      <c r="H18" s="7" t="inlineStr">
+      <c r="H17" s="7" t="inlineStr">
         <is>
           <t>Not linked yet</t>
         </is>
       </c>
-      <c r="I18" s="5" t="inlineStr">
+      <c r="I17" s="5" t="inlineStr">
         <is>
           <t>Draft</t>
         </is>
       </c>
-      <c r="J18" s="6" t="inlineStr">
+      <c r="J17" s="6" t="inlineStr">
         <is>
           <t>my best run today. someone's already ahead of it 😭 same seed, same day, go beat them. link in bio</t>
         </is>
       </c>
-      <c r="K18" s="5" t="inlineStr">
+      <c r="K17" s="5" t="inlineStr">
         <is>
           <t>#dailychallenge #indiegame #gamingmemes #leaderboard</t>
         </is>
       </c>
-      <c r="L18" s="6" t="inlineStr">
+      <c r="L17" s="6" t="inlineStr">
         <is>
           <t>my best today. this guy's best today 💀 same run, same day, link in bio</t>
         </is>
       </c>
-      <c r="M18" s="6" t="inlineStr"/>
-      <c r="N18" s="5" t="inlineStr">
+      <c r="M17" s="6" t="inlineStr"/>
+      <c r="N17" s="5" t="inlineStr">
         <is>
           <t>Someone Already Beat My Best Run Today (ORION)</t>
         </is>
       </c>
-      <c r="O18" s="6" t="inlineStr">
+      <c r="O17" s="6" t="inlineStr">
         <is>
           <t>Same seed as every pilot. The board never sits still. Free dodging game, three attempts a day.
 Play: https://surviveorion.com
@@ -1787,70 +1716,70 @@
         </is>
       </c>
     </row>
-    <row r="19" ht="60" customHeight="1">
-      <c r="A19" s="5" t="inlineStr">
+    <row r="18" ht="60" customHeight="1">
+      <c r="A18" s="5" t="inlineStr">
         <is>
           <t>2026-09-05</t>
         </is>
       </c>
-      <c r="B19" s="5" t="inlineStr">
+      <c r="B18" s="5" t="inlineStr">
         <is>
           <t>Sat</t>
         </is>
       </c>
-      <c r="C19" s="5" t="inlineStr">
+      <c r="C18" s="5" t="inlineStr">
         <is>
           <t>TODAY'S PATROL</t>
         </is>
       </c>
-      <c r="D19" s="5" t="inlineStr">
+      <c r="D18" s="5" t="inlineStr">
         <is>
           <t>YEAR OF THE SERPENT</t>
         </is>
       </c>
-      <c r="E19" s="6" t="inlineStr">
+      <c r="E18" s="6" t="inlineStr">
         <is>
           <t>Every formation slithers today. Watch the trains.</t>
         </is>
       </c>
-      <c r="F19" s="5" t="n"/>
-      <c r="G19" s="5" t="inlineStr">
+      <c r="F18" s="5" t="n"/>
+      <c r="G18" s="5" t="inlineStr">
         <is>
           <t>0905_patrol_yearoftheserpent_916.mov</t>
         </is>
       </c>
-      <c r="H19" s="7" t="inlineStr">
+      <c r="H18" s="7" t="inlineStr">
         <is>
           <t>Not linked yet</t>
         </is>
       </c>
-      <c r="I19" s="5" t="inlineStr">
+      <c r="I18" s="5" t="inlineStr">
         <is>
           <t>Draft</t>
         </is>
       </c>
-      <c r="J19" s="6" t="inlineStr">
+      <c r="J18" s="6" t="inlineStr">
         <is>
           <t>Today every pilot flies YEAR OF THE SERPENT: Every formation slithers today. Watch the trains. Three attempts. Free, in your browser.</t>
         </is>
       </c>
-      <c r="K19" s="5" t="inlineStr">
+      <c r="K18" s="5" t="inlineStr">
         <is>
           <t>#dailychallenge #indiegame #browsergame #arcadegame</t>
         </is>
       </c>
-      <c r="L19" s="6" t="inlineStr">
+      <c r="L18" s="6" t="inlineStr">
         <is>
           <t>today every pilot flies year of the serpent: every formation slithers today. watch the trains. three attempts. free, in your browser.</t>
         </is>
       </c>
-      <c r="M19" s="6" t="n"/>
-      <c r="N19" s="5" t="inlineStr">
+      <c r="M18" s="6" t="n"/>
+      <c r="N18" s="5" t="inlineStr">
         <is>
           <t>YEAR OF THE SERPENT DAY: Today's ORION Patrol (Day 54)</t>
         </is>
       </c>
-      <c r="O19" s="6" t="inlineStr">
+      <c r="O18" s="6" t="inlineStr">
         <is>
           <t>Today's shared seed: YEAR OF THE SERPENT. No ambient drones at all. Only serpent trains, more of them, released to hunt after their sweep. Deep in the run the trains keep coming faster and stray drones start leaking in. Every pilot flies the same run. Three attempts, free in your browser.
 Play now: https://surviveorion.com
@@ -1858,74 +1787,74 @@
         </is>
       </c>
     </row>
-    <row r="20" ht="60" customHeight="1">
-      <c r="A20" s="5" t="inlineStr">
+    <row r="19" ht="60" customHeight="1">
+      <c r="A19" s="5" t="inlineStr">
         <is>
           <t>2026-09-06</t>
         </is>
       </c>
-      <c r="B20" s="5" t="inlineStr">
+      <c r="B19" s="5" t="inlineStr">
         <is>
           <t>Sun</t>
         </is>
       </c>
-      <c r="C20" s="5" t="inlineStr">
+      <c r="C19" s="5" t="inlineStr">
         <is>
           <t>TODAY'S PATROL · SUNDAY DOUBLE</t>
         </is>
       </c>
-      <c r="D20" s="5" t="inlineStr">
+      <c r="D19" s="5" t="inlineStr">
         <is>
           <t>PATROL: MAGNETIC FIELD + CLOAK</t>
         </is>
       </c>
-      <c r="E20" s="6" t="inlineStr">
+      <c r="E19" s="6" t="inlineStr">
         <is>
           <t>The pickups want to find you today. They lose the lock. You seed the dark.</t>
         </is>
       </c>
-      <c r="F20" s="5" t="inlineStr">
+      <c r="F19" s="5" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="G20" s="5" t="inlineStr">
+      <c r="G19" s="5" t="inlineStr">
         <is>
           <t>0906_patrol_magneticfieldcloak_916.mov</t>
         </is>
       </c>
-      <c r="H20" s="7" t="inlineStr">
+      <c r="H19" s="7" t="inlineStr">
         <is>
           <t>Not linked yet</t>
         </is>
       </c>
-      <c r="I20" s="5" t="inlineStr">
+      <c r="I19" s="5" t="inlineStr">
         <is>
           <t>Draft</t>
         </is>
       </c>
-      <c r="J20" s="6" t="inlineStr">
+      <c r="J19" s="6" t="inlineStr">
         <is>
           <t>Today every pilot flies MAGNETIC FIELD + CLOAK: The pickups want to find you today. They lose the lock. You seed the dark. Three attempts. Free, in your browser.</t>
         </is>
       </c>
-      <c r="K20" s="5" t="inlineStr">
+      <c r="K19" s="5" t="inlineStr">
         <is>
           <t>#dailychallenge #indiegame #browsergame #arcadegame</t>
         </is>
       </c>
-      <c r="L20" s="6" t="inlineStr">
+      <c r="L19" s="6" t="inlineStr">
         <is>
           <t>today every pilot flies magnetic field + cloak: the pickups want to find you today. they lose the lock. you seed the dark. three attempts. free, in your browser.</t>
         </is>
       </c>
-      <c r="M20" s="6" t="n"/>
-      <c r="N20" s="5" t="inlineStr">
+      <c r="M19" s="6" t="n"/>
+      <c r="N19" s="5" t="inlineStr">
         <is>
           <t>MAGNETIC FIELD + CLOAK DAY: Today's ORION Patrol (Day 55)</t>
         </is>
       </c>
-      <c r="O20" s="6" t="inlineStr">
+      <c r="O19" s="6" t="inlineStr">
         <is>
           <t>Today's shared seed: MAGNETIC FIELD + CLOAK. Pickups slowly drift toward your ship all day, on top of their normal wander. Every pickup is Cloak. Drones hover, lost. Invisible bombs drop along your path and explode when you reappear. Every pilot flies the same run. Three attempts, free in your browser.
 Play now: https://surviveorion.com
@@ -1933,70 +1862,70 @@
         </is>
       </c>
     </row>
-    <row r="21" ht="60" customHeight="1">
-      <c r="A21" s="5" t="inlineStr">
+    <row r="20" ht="60" customHeight="1">
+      <c r="A20" s="5" t="inlineStr">
         <is>
           <t>2026-09-07</t>
         </is>
       </c>
-      <c r="B21" s="5" t="inlineStr">
+      <c r="B20" s="5" t="inlineStr">
         <is>
           <t>Mon</t>
         </is>
       </c>
-      <c r="C21" s="5" t="inlineStr">
+      <c r="C20" s="5" t="inlineStr">
         <is>
           <t>BUG</t>
         </is>
       </c>
-      <c r="D21" s="5" t="inlineStr">
+      <c r="D20" s="5" t="inlineStr">
         <is>
           <t>Bug of the week</t>
         </is>
       </c>
-      <c r="E21" s="6" t="inlineStr">
+      <c r="E20" s="6" t="inlineStr">
         <is>
           <t>Any real glitch, physics jank, or weird interaction. Film it as-is, matter-of-fact caption, no apology. "Who needs new features when you got old bugs."</t>
         </is>
       </c>
-      <c r="F21" s="5" t="inlineStr"/>
-      <c r="G21" s="5" t="inlineStr">
+      <c r="F20" s="5" t="inlineStr"/>
+      <c r="G20" s="5" t="inlineStr">
         <is>
           <t>0907_bugoftheweek_916.mov</t>
         </is>
       </c>
-      <c r="H21" s="7" t="inlineStr">
+      <c r="H20" s="7" t="inlineStr">
         <is>
           <t>Not linked yet</t>
         </is>
       </c>
-      <c r="I21" s="5" t="inlineStr">
+      <c r="I20" s="5" t="inlineStr">
         <is>
           <t>Draft</t>
         </is>
       </c>
-      <c r="J21" s="6" t="inlineStr">
+      <c r="J20" s="6" t="inlineStr">
         <is>
           <t>bug of the week. we see it too. free browser game, link in bio</t>
         </is>
       </c>
-      <c r="K21" s="5" t="inlineStr">
+      <c r="K20" s="5" t="inlineStr">
         <is>
           <t>#gamedev #indiegame #gamingmemes #bug</t>
         </is>
       </c>
-      <c r="L21" s="6" t="inlineStr">
+      <c r="L20" s="6" t="inlineStr">
         <is>
           <t>bug of the week 💀 nobody's perfect, free daily dodge game, link in bio</t>
         </is>
       </c>
-      <c r="M21" s="6" t="inlineStr"/>
-      <c r="N21" s="5" t="inlineStr">
+      <c r="M20" s="6" t="inlineStr"/>
+      <c r="N20" s="5" t="inlineStr">
         <is>
           <t>Bug of the Week (ORION Devlog Clip)</t>
         </is>
       </c>
-      <c r="O21" s="6" t="inlineStr">
+      <c r="O20" s="6" t="inlineStr">
         <is>
           <t>Real jank, filmed as it happened. Free daily dodging game.
 Play: https://surviveorion.com
@@ -2004,70 +1933,70 @@
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="5" t="inlineStr">
+    <row r="21" ht="60" customHeight="1">
+      <c r="A21" s="5" t="inlineStr">
         <is>
           <t>2026-09-07</t>
         </is>
       </c>
-      <c r="B22" s="5" t="inlineStr">
+      <c r="B21" s="5" t="inlineStr">
         <is>
           <t>Mon</t>
         </is>
       </c>
-      <c r="C22" s="5" t="inlineStr">
+      <c r="C21" s="5" t="inlineStr">
         <is>
           <t>TODAY'S PATROL</t>
         </is>
       </c>
-      <c r="D22" s="5" t="inlineStr">
+      <c r="D21" s="5" t="inlineStr">
         <is>
           <t>RAM RAID</t>
         </is>
       </c>
-      <c r="E22" s="6" t="inlineStr">
+      <c r="E21" s="6" t="inlineStr">
         <is>
           <t>The shell is short. Spend it, then dodge naked.</t>
         </is>
       </c>
-      <c r="F22" s="5" t="n"/>
-      <c r="G22" s="5" t="inlineStr">
+      <c r="F21" s="5" t="n"/>
+      <c r="G21" s="5" t="inlineStr">
         <is>
           <t>0907_patrol_ramraid_916.mov</t>
         </is>
       </c>
-      <c r="H22" s="7" t="inlineStr">
+      <c r="H21" s="7" t="inlineStr">
         <is>
           <t>Not linked yet</t>
         </is>
       </c>
-      <c r="I22" s="5" t="inlineStr">
+      <c r="I21" s="5" t="inlineStr">
         <is>
           <t>Draft</t>
         </is>
       </c>
-      <c r="J22" s="6" t="inlineStr">
+      <c r="J21" s="6" t="inlineStr">
         <is>
           <t>Today every pilot flies RAM RAID: The shell is short. Spend it, then dodge naked. Three attempts. Free, in your browser.</t>
         </is>
       </c>
-      <c r="K22" s="5" t="inlineStr">
+      <c r="K21" s="5" t="inlineStr">
         <is>
           <t>#dailychallenge #indiegame #browsergame #arcadegame</t>
         </is>
       </c>
-      <c r="L22" s="6" t="inlineStr">
+      <c r="L21" s="6" t="inlineStr">
         <is>
           <t>today every pilot flies ram raid: the shell is short. spend it, then dodge naked. three attempts. free, in your browser.</t>
         </is>
       </c>
-      <c r="M22" s="6" t="n"/>
-      <c r="N22" s="5" t="inlineStr">
+      <c r="M21" s="6" t="n"/>
+      <c r="N21" s="5" t="inlineStr">
         <is>
           <t>RAM RAID DAY: Today's ORION Patrol (Day 56)</t>
         </is>
       </c>
-      <c r="O22" s="6" t="inlineStr">
+      <c r="O21" s="6" t="inlineStr">
         <is>
           <t>Today's shared seed: RAM RAID. Starshell is the only drop, and it is scarce. The shell lasts about two seconds. You are invincible while it is up. Every pilot flies the same run. Three attempts, free in your browser.
 Play now: https://surviveorion.com
@@ -2075,70 +2004,70 @@
         </is>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" s="5" t="inlineStr">
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
         <is>
           <t>2026-09-08</t>
         </is>
       </c>
-      <c r="B23" s="5" t="inlineStr">
+      <c r="B22" s="5" t="inlineStr">
         <is>
           <t>Tue</t>
         </is>
       </c>
-      <c r="C23" s="5" t="inlineStr">
+      <c r="C22" s="5" t="inlineStr">
         <is>
           <t>TODAY'S PATROL</t>
         </is>
       </c>
-      <c r="D23" s="5" t="inlineStr">
+      <c r="D22" s="5" t="inlineStr">
         <is>
           <t>SINGULARITY</t>
         </is>
       </c>
-      <c r="E23" s="6" t="inlineStr">
+      <c r="E22" s="6" t="inlineStr">
         <is>
           <t>The banned singularity is back for one day. Use it well.</t>
         </is>
       </c>
-      <c r="F23" s="5" t="n"/>
-      <c r="G23" s="5" t="inlineStr">
+      <c r="F22" s="5" t="n"/>
+      <c r="G22" s="5" t="inlineStr">
         <is>
           <t>0908_patrol_singularity_916.mov</t>
         </is>
       </c>
-      <c r="H23" s="7" t="inlineStr">
+      <c r="H22" s="7" t="inlineStr">
         <is>
           <t>Not linked yet</t>
         </is>
       </c>
-      <c r="I23" s="5" t="inlineStr">
+      <c r="I22" s="5" t="inlineStr">
         <is>
           <t>Draft</t>
         </is>
       </c>
-      <c r="J23" s="6" t="inlineStr">
+      <c r="J22" s="6" t="inlineStr">
         <is>
           <t>Today every pilot flies SINGULARITY: The banned singularity is back for one day. Use it well. Three attempts. Free, in your browser.</t>
         </is>
       </c>
-      <c r="K23" s="5" t="inlineStr">
+      <c r="K22" s="5" t="inlineStr">
         <is>
           <t>#dailychallenge #indiegame #browsergame #arcadegame</t>
         </is>
       </c>
-      <c r="L23" s="6" t="inlineStr">
+      <c r="L22" s="6" t="inlineStr">
         <is>
           <t>today every pilot flies singularity: the banned singularity is back for one day. use it well. three attempts. free, in your browser.</t>
         </is>
       </c>
-      <c r="M23" s="6" t="n"/>
-      <c r="N23" s="5" t="inlineStr">
+      <c r="M22" s="6" t="n"/>
+      <c r="N22" s="5" t="inlineStr">
         <is>
           <t>SINGULARITY DAY: Today's ORION Patrol (Day 57)</t>
         </is>
       </c>
-      <c r="O23" s="6" t="inlineStr">
+      <c r="O22" s="6" t="inlineStr">
         <is>
           <t>Today's shared seed: SINGULARITY. Vortex (normally benched) drops often today. Every pilot flies the same run. Three attempts, free in your browser.
 Play now: https://surviveorion.com
@@ -2146,68 +2075,68 @@
         </is>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
+    <row r="23">
+      <c r="A23" t="inlineStr">
         <is>
           <t>2026-09-26</t>
         </is>
       </c>
-      <c r="B24" t="inlineStr">
+      <c r="B23" t="inlineStr">
         <is>
           <t>Sat</t>
         </is>
       </c>
-      <c r="C24" t="inlineStr">
+      <c r="C23" t="inlineStr">
         <is>
           <t>TODAY'S PATROL</t>
         </is>
       </c>
-      <c r="D24" t="inlineStr">
+      <c r="D23" t="inlineStr">
         <is>
           <t>GREAT WALL</t>
         </is>
       </c>
-      <c r="E24" t="inlineStr">
+      <c r="E23" t="inlineStr">
         <is>
           <t>nothing but walls today.</t>
         </is>
       </c>
-      <c r="G24" t="inlineStr">
+      <c r="G23" t="inlineStr">
         <is>
           <t>0827_greatwall_916.mov</t>
         </is>
       </c>
-      <c r="H24" t="inlineStr">
+      <c r="H23" t="inlineStr">
         <is>
           <t>Linked</t>
         </is>
       </c>
-      <c r="I24" t="inlineStr">
+      <c r="I23" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
       </c>
-      <c r="J24" t="inlineStr">
+      <c r="J23" t="inlineStr">
         <is>
           <t>Today every pilot flies GREAT WALL: nothing but walls today. Three attempts. Free, in your browser.</t>
         </is>
       </c>
-      <c r="K24" t="inlineStr">
+      <c r="K23" t="inlineStr">
         <is>
           <t>#dailychallenge #indiegame #browsergame #arcadegame</t>
         </is>
       </c>
-      <c r="L24" t="inlineStr">
+      <c r="L23" t="inlineStr">
         <is>
           <t>today every pilot flies great wall: nothing but walls today. three attempts. free, in your browser.</t>
         </is>
       </c>
-      <c r="N24" t="inlineStr">
+      <c r="N23" t="inlineStr">
         <is>
           <t>GREAT WALL DAY: Today's ORION Patrol (Day 75)</t>
         </is>
       </c>
-      <c r="O24" t="inlineStr">
+      <c r="O23" t="inlineStr">
         <is>
           <t>Today's shared seed: GREAT WALL. No ambient drones at all. Only walls, mega walls, and pincers, faster than usual, released to hunt after their sweep. Every pilot flies the same run. Three attempts, free in your browser.
 Play now: https://surviveorion.com

</xml_diff>

<commit_message>
Host Ditch the Can and Dead Fart, with copy from the on-video hooks.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/ORION_Publishing_Calendar.xlsx
+++ b/ORION_Publishing_Calendar.xlsx
@@ -487,7 +487,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O23"/>
+  <dimension ref="A1:O25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -1291,10 +1291,8 @@
       </c>
     </row>
     <row r="12" ht="60" customHeight="1">
-      <c r="A12" s="5" t="inlineStr">
-        <is>
-          <t>2026-09-01</t>
-        </is>
+      <c r="A12" s="8" t="n">
+        <v>46266</v>
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
@@ -1303,57 +1301,128 @@
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>TODAY'S PATROL</t>
+          <t>POV</t>
         </is>
       </c>
       <c r="D12" s="5" t="inlineStr">
         <is>
-          <t>STARFALL</t>
+          <t>Ditch the Can</t>
         </is>
       </c>
       <c r="E12" s="6" t="inlineStr">
         <is>
-          <t>The sky opens early. Shields are scarce.</t>
+          <t>Bored? Ditch the can</t>
         </is>
       </c>
       <c r="F12" s="5" t="n"/>
       <c r="G12" s="5" t="inlineStr">
         <is>
-          <t>0901_patrol_starfall_916.mov</t>
+          <t>0828_ditchthecan_916.mp4</t>
         </is>
       </c>
       <c r="H12" s="7" t="inlineStr">
         <is>
-          <t>Not linked yet</t>
+          <t>Linked</t>
         </is>
       </c>
       <c r="I12" s="5" t="inlineStr">
         <is>
-          <t>Draft</t>
+          <t>Approved</t>
         </is>
       </c>
       <c r="J12" s="6" t="inlineStr">
         <is>
-          <t>Today every pilot flies STARFALL: The sky opens early. Shields are scarce. Three attempts. Free, in your browser.</t>
+          <t>Bored? Ditch the can. Play ORION instead 🛰️ Daily dodge, three attempts, free. Link in bio.</t>
         </is>
       </c>
       <c r="K12" s="5" t="inlineStr">
         <is>
-          <t>#dailychallenge #indiegame #browsergame #arcadegame</t>
+          <t>#gamingmemes #indiegame #dailychallenge #browsergame</t>
         </is>
       </c>
       <c r="L12" s="6" t="inlineStr">
         <is>
-          <t>today every pilot flies starfall: the sky opens early. shields are scarce. three attempts. free, in your browser.</t>
+          <t>bored? ditch the can. play orion instead 💀 free daily dodge game, 3 attempts, link in bio</t>
         </is>
       </c>
       <c r="M12" s="6" t="n"/>
       <c r="N12" s="5" t="inlineStr">
         <is>
+          <t>Bored? Ditch the Can. Play ORION Instead</t>
+        </is>
+      </c>
+      <c r="O12" s="6" t="inlineStr">
+        <is>
+          <t>Reading the can again? Daily dodge game. Three attempts, same run as every other pilot. It's free.
+Play: https://surviveorion.com
+#gamingmemes #indiegame #Shorts</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="60" customHeight="1">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>Tue</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>TODAY'S PATROL</t>
+        </is>
+      </c>
+      <c r="D13" s="5" t="inlineStr">
+        <is>
+          <t>STARFALL</t>
+        </is>
+      </c>
+      <c r="E13" s="6" t="inlineStr">
+        <is>
+          <t>The sky opens early. Shields are scarce.</t>
+        </is>
+      </c>
+      <c r="F13" s="5" t="n"/>
+      <c r="G13" s="5" t="inlineStr">
+        <is>
+          <t>0901_patrol_starfall_916.mov</t>
+        </is>
+      </c>
+      <c r="H13" s="7" t="inlineStr">
+        <is>
+          <t>Not linked yet</t>
+        </is>
+      </c>
+      <c r="I13" s="5" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="J13" s="6" t="inlineStr">
+        <is>
+          <t>Today every pilot flies STARFALL: The sky opens early. Shields are scarce. Three attempts. Free, in your browser.</t>
+        </is>
+      </c>
+      <c r="K13" s="5" t="inlineStr">
+        <is>
+          <t>#dailychallenge #indiegame #browsergame #arcadegame</t>
+        </is>
+      </c>
+      <c r="L13" s="6" t="inlineStr">
+        <is>
+          <t>today every pilot flies starfall: the sky opens early. shields are scarce. three attempts. free, in your browser.</t>
+        </is>
+      </c>
+      <c r="M13" s="6" t="n"/>
+      <c r="N13" s="5" t="inlineStr">
+        <is>
           <t>STARFALL DAY: Today's ORION Patrol (Day 50)</t>
         </is>
       </c>
-      <c r="O12" s="6" t="inlineStr">
+      <c r="O13" s="6" t="inlineStr">
         <is>
           <t>Today's shared seed: STARFALL. Meteor rain from the first seconds. Shield is the only drop, and it is late. Every pilot flies the same run. Three attempts, free in your browser.
 Play now: https://surviveorion.com
@@ -1361,70 +1430,139 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="60" customHeight="1">
-      <c r="A13" s="5" t="inlineStr">
+    <row r="14" ht="60" customHeight="1">
+      <c r="A14" s="8" t="n">
+        <v>46267</v>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>Wed</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>SPACE DUST</t>
+        </is>
+      </c>
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>Dead Fart</t>
+        </is>
+      </c>
+      <c r="E14" s="6" t="inlineStr">
+        <is>
+          <t>he died. the game farted.</t>
+        </is>
+      </c>
+      <c r="F14" s="5" t="n"/>
+      <c r="G14" s="5" t="inlineStr">
+        <is>
+          <t>0828_deadfartsound_916.mp4</t>
+        </is>
+      </c>
+      <c r="H14" s="7" t="inlineStr">
+        <is>
+          <t>Linked</t>
+        </is>
+      </c>
+      <c r="I14" s="5" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="J14" s="6" t="inlineStr">
+        <is>
+          <t>he died. the game farted. 💀 Free daily dodge game, link in bio.</t>
+        </is>
+      </c>
+      <c r="K14" s="5" t="inlineStr">
+        <is>
+          <t>#gamingmemes #indiegame #fail #dailychallenge #browsergame</t>
+        </is>
+      </c>
+      <c r="L14" s="6" t="inlineStr">
+        <is>
+          <t>he died. the game farted. 💀 free daily dodge game, 3 attempts, link in bio</t>
+        </is>
+      </c>
+      <c r="M14" s="6" t="n"/>
+      <c r="N14" s="5" t="inlineStr">
+        <is>
+          <t>He Died. The Game Farted. (ORION)</t>
+        </is>
+      </c>
+      <c r="O14" s="6" t="inlineStr">
+        <is>
+          <t>The daily patrol remains undefeated. The sound design had opinions.
+Play: https://surviveorion.com
+#Shorts</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="60" customHeight="1">
+      <c r="A15" s="5" t="inlineStr">
         <is>
           <t>2026-09-02</t>
         </is>
       </c>
-      <c r="B13" s="5" t="inlineStr">
+      <c r="B15" s="5" t="inlineStr">
         <is>
           <t>Wed</t>
         </is>
       </c>
-      <c r="C13" s="5" t="inlineStr">
+      <c r="C15" s="5" t="inlineStr">
         <is>
           <t>TODAY'S PATROL</t>
         </is>
       </c>
-      <c r="D13" s="5" t="inlineStr">
+      <c r="D15" s="5" t="inlineStr">
         <is>
           <t>RED ALERT</t>
         </is>
       </c>
-      <c r="E13" s="6" t="inlineStr">
+      <c r="E15" s="6" t="inlineStr">
         <is>
           <t>Klaxons up. Everything moves faster except you.</t>
         </is>
       </c>
-      <c r="F13" s="5" t="n"/>
-      <c r="G13" s="5" t="inlineStr">
+      <c r="F15" s="5" t="n"/>
+      <c r="G15" s="5" t="inlineStr">
         <is>
           <t>0902_patrol_redalert_916.mov</t>
         </is>
       </c>
-      <c r="H13" s="7" t="inlineStr">
+      <c r="H15" s="7" t="inlineStr">
         <is>
           <t>Not linked yet</t>
         </is>
       </c>
-      <c r="I13" s="5" t="inlineStr">
+      <c r="I15" s="5" t="inlineStr">
         <is>
           <t>Draft</t>
         </is>
       </c>
-      <c r="J13" s="6" t="inlineStr">
+      <c r="J15" s="6" t="inlineStr">
         <is>
           <t>Today every pilot flies RED ALERT: Klaxons up. Everything moves faster except you. Three attempts. Free, in your browser.</t>
         </is>
       </c>
-      <c r="K13" s="5" t="inlineStr">
+      <c r="K15" s="5" t="inlineStr">
         <is>
           <t>#dailychallenge #indiegame #browsergame #arcadegame</t>
         </is>
       </c>
-      <c r="L13" s="6" t="inlineStr">
+      <c r="L15" s="6" t="inlineStr">
         <is>
           <t>today every pilot flies red alert: klaxons up. everything moves faster except you. three attempts. free, in your browser.</t>
         </is>
       </c>
-      <c r="M13" s="6" t="n"/>
-      <c r="N13" s="5" t="inlineStr">
+      <c r="M15" s="6" t="n"/>
+      <c r="N15" s="5" t="inlineStr">
         <is>
           <t>RED ALERT DAY: Today's ORION Patrol (Day 51)</t>
         </is>
       </c>
-      <c r="O13" s="6" t="inlineStr">
+      <c r="O15" s="6" t="inlineStr">
         <is>
           <t>Today's shared seed: RED ALERT. Spawn rate, formation frequency, and pickup drops all sped up. Drone speed is unchanged. Every pilot flies the same run. Three attempts, free in your browser.
 Play now: https://surviveorion.com
@@ -1432,70 +1570,70 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="60" customHeight="1">
-      <c r="A14" s="5" t="inlineStr">
+    <row r="16" ht="60" customHeight="1">
+      <c r="A16" s="5" t="inlineStr">
         <is>
           <t>2026-09-03</t>
         </is>
       </c>
-      <c r="B14" s="5" t="inlineStr">
+      <c r="B16" s="5" t="inlineStr">
         <is>
           <t>Thu</t>
         </is>
       </c>
-      <c r="C14" s="5" t="inlineStr">
+      <c r="C16" s="5" t="inlineStr">
         <is>
           <t>NEW BEST</t>
         </is>
       </c>
-      <c r="D14" s="5" t="inlineStr">
+      <c r="D16" s="5" t="inlineStr">
         <is>
           <t>NEW BEST</t>
         </is>
       </c>
-      <c r="E14" s="6" t="inlineStr">
+      <c r="E16" s="6" t="inlineStr">
         <is>
           <t>Any run that beats your HUD best. The in-app celebration sound is already the hook, cut around it.</t>
         </is>
       </c>
-      <c r="F14" s="5" t="inlineStr"/>
-      <c r="G14" s="5" t="inlineStr">
+      <c r="F16" s="5" t="inlineStr"/>
+      <c r="G16" s="5" t="inlineStr">
         <is>
           <t>0903_newbest_916.mov</t>
         </is>
       </c>
-      <c r="H14" s="7" t="inlineStr">
+      <c r="H16" s="7" t="inlineStr">
         <is>
           <t>Not linked yet</t>
         </is>
       </c>
-      <c r="I14" s="5" t="inlineStr">
+      <c r="I16" s="5" t="inlineStr">
         <is>
           <t>Draft</t>
         </is>
       </c>
-      <c r="J14" s="6" t="inlineStr">
+      <c r="J16" s="6" t="inlineStr">
         <is>
           <t>new personal best 🏆 same run as every other pilot today. free browser game, link in bio</t>
         </is>
       </c>
-      <c r="K14" s="5" t="inlineStr">
+      <c r="K16" s="5" t="inlineStr">
         <is>
           <t>#indiegame #gamingmemes #personalbest #dailychallenge</t>
         </is>
       </c>
-      <c r="L14" s="6" t="inlineStr">
+      <c r="L16" s="6" t="inlineStr">
         <is>
           <t>new best 🏆 free daily dodge game, link in bio</t>
         </is>
       </c>
-      <c r="M14" s="6" t="inlineStr"/>
-      <c r="N14" s="5" t="inlineStr">
+      <c r="M16" s="6" t="inlineStr"/>
+      <c r="N16" s="5" t="inlineStr">
         <is>
           <t>New Personal Best (ORION Daily Patrol)</t>
         </is>
       </c>
-      <c r="O14" s="6" t="inlineStr">
+      <c r="O16" s="6" t="inlineStr">
         <is>
           <t>Same seed as every pilot today. Free dodging game, three attempts a day.
 Play: https://surviveorion.com
@@ -1503,70 +1641,70 @@
         </is>
       </c>
     </row>
-    <row r="15" ht="60" customHeight="1">
-      <c r="A15" s="5" t="inlineStr">
+    <row r="17" ht="60" customHeight="1">
+      <c r="A17" s="5" t="inlineStr">
         <is>
           <t>2026-09-03</t>
         </is>
       </c>
-      <c r="B15" s="5" t="inlineStr">
+      <c r="B17" s="5" t="inlineStr">
         <is>
           <t>Thu</t>
         </is>
       </c>
-      <c r="C15" s="5" t="inlineStr">
+      <c r="C17" s="5" t="inlineStr">
         <is>
           <t>TODAY'S PATROL</t>
         </is>
       </c>
-      <c r="D15" s="5" t="inlineStr">
+      <c r="D17" s="5" t="inlineStr">
         <is>
           <t>THE FLOOD</t>
         </is>
       </c>
-      <c r="E15" s="6" t="inlineStr">
+      <c r="E17" s="6" t="inlineStr">
         <is>
           <t>No formations. They just keep popping in.</t>
         </is>
       </c>
-      <c r="F15" s="5" t="n"/>
-      <c r="G15" s="5" t="inlineStr">
+      <c r="F17" s="5" t="n"/>
+      <c r="G17" s="5" t="inlineStr">
         <is>
           <t>0903_patrol_theflood_916.mov</t>
         </is>
       </c>
-      <c r="H15" s="7" t="inlineStr">
+      <c r="H17" s="7" t="inlineStr">
         <is>
           <t>Not linked yet</t>
         </is>
       </c>
-      <c r="I15" s="5" t="inlineStr">
+      <c r="I17" s="5" t="inlineStr">
         <is>
           <t>Draft</t>
         </is>
       </c>
-      <c r="J15" s="6" t="inlineStr">
+      <c r="J17" s="6" t="inlineStr">
         <is>
           <t>Today every pilot flies THE FLOOD: No formations. They just keep popping in. Three attempts. Free, in your browser.</t>
         </is>
       </c>
-      <c r="K15" s="5" t="inlineStr">
+      <c r="K17" s="5" t="inlineStr">
         <is>
           <t>#dailychallenge #indiegame #browsergame #arcadegame</t>
         </is>
       </c>
-      <c r="L15" s="6" t="inlineStr">
+      <c r="L17" s="6" t="inlineStr">
         <is>
           <t>today every pilot flies the flood: no formations. they just keep popping in. three attempts. free, in your browser.</t>
         </is>
       </c>
-      <c r="M15" s="6" t="n"/>
-      <c r="N15" s="5" t="inlineStr">
+      <c r="M17" s="6" t="n"/>
+      <c r="N17" s="5" t="inlineStr">
         <is>
           <t>THE FLOOD DAY: Today's ORION Patrol (Day 52)</t>
         </is>
       </c>
-      <c r="O15" s="6" t="inlineStr">
+      <c r="O17" s="6" t="inlineStr">
         <is>
           <t>Today's shared seed: THE FLOOD. A constant beat from the edges. The beat speeds up the whole run. Every pilot flies the same run. Three attempts, free in your browser.
 Play now: https://surviveorion.com
@@ -1574,70 +1712,70 @@
         </is>
       </c>
     </row>
-    <row r="16" ht="60" customHeight="1">
-      <c r="A16" s="5" t="inlineStr">
+    <row r="18" ht="60" customHeight="1">
+      <c r="A18" s="5" t="inlineStr">
         <is>
           <t>2026-09-04</t>
         </is>
       </c>
-      <c r="B16" s="5" t="inlineStr">
+      <c r="B18" s="5" t="inlineStr">
         <is>
           <t>Fri</t>
         </is>
       </c>
-      <c r="C16" s="5" t="inlineStr">
+      <c r="C18" s="5" t="inlineStr">
         <is>
           <t>TODAY'S PATROL</t>
         </is>
       </c>
-      <c r="D16" s="5" t="inlineStr">
+      <c r="D18" s="5" t="inlineStr">
         <is>
           <t>THUNDER</t>
         </is>
       </c>
-      <c r="E16" s="6" t="inlineStr">
+      <c r="E18" s="6" t="inlineStr">
         <is>
           <t>Aim the ray. Let it hop.</t>
         </is>
       </c>
-      <c r="F16" s="5" t="n"/>
-      <c r="G16" s="5" t="inlineStr">
+      <c r="F18" s="5" t="n"/>
+      <c r="G18" s="5" t="inlineStr">
         <is>
           <t>0904_patrol_thunder_916.mov</t>
         </is>
       </c>
-      <c r="H16" s="7" t="inlineStr">
+      <c r="H18" s="7" t="inlineStr">
         <is>
           <t>Not linked yet</t>
         </is>
       </c>
-      <c r="I16" s="5" t="inlineStr">
+      <c r="I18" s="5" t="inlineStr">
         <is>
           <t>Draft</t>
         </is>
       </c>
-      <c r="J16" s="6" t="inlineStr">
+      <c r="J18" s="6" t="inlineStr">
         <is>
           <t>Today every pilot flies THUNDER: Aim the ray. Let it hop. Three attempts. Free, in your browser.</t>
         </is>
       </c>
-      <c r="K16" s="5" t="inlineStr">
+      <c r="K18" s="5" t="inlineStr">
         <is>
           <t>#dailychallenge #indiegame #browsergame #arcadegame</t>
         </is>
       </c>
-      <c r="L16" s="6" t="inlineStr">
+      <c r="L18" s="6" t="inlineStr">
         <is>
           <t>today every pilot flies thunder: aim the ray. let it hop. three attempts. free, in your browser.</t>
         </is>
       </c>
-      <c r="M16" s="6" t="n"/>
-      <c r="N16" s="5" t="inlineStr">
+      <c r="M18" s="6" t="n"/>
+      <c r="N18" s="5" t="inlineStr">
         <is>
           <t>THUNDER DAY: Today's ORION Patrol (Day 53)</t>
         </is>
       </c>
-      <c r="O16" s="6" t="inlineStr">
+      <c r="O18" s="6" t="inlineStr">
         <is>
           <t>Today's shared seed: THUNDER. Every pickup is Thunder. A lightning ray along your nose. Each kill sparks Arc hops. Ray kills pay double. Every pilot flies the same run. Three attempts, free in your browser.
 Play now: https://surviveorion.com
@@ -1645,70 +1783,70 @@
         </is>
       </c>
     </row>
-    <row r="17" ht="60" customHeight="1">
-      <c r="A17" s="5" t="inlineStr">
+    <row r="19" ht="60" customHeight="1">
+      <c r="A19" s="5" t="inlineStr">
         <is>
           <t>2026-09-05</t>
         </is>
       </c>
-      <c r="B17" s="5" t="inlineStr">
+      <c r="B19" s="5" t="inlineStr">
         <is>
           <t>Sat</t>
         </is>
       </c>
-      <c r="C17" s="5" t="inlineStr">
+      <c r="C19" s="5" t="inlineStr">
         <is>
           <t>THE BOARD</t>
         </is>
       </c>
-      <c r="D17" s="5" t="inlineStr">
+      <c r="D19" s="5" t="inlineStr">
         <is>
           <t>Beaten by a stranger</t>
         </is>
       </c>
-      <c r="E17" s="6" t="inlineStr">
+      <c r="E19" s="6" t="inlineStr">
         <is>
           <t>Your best run of the day, then the board showing someone above you right now. Ends on the gap, not the score.</t>
         </is>
       </c>
-      <c r="F17" s="5" t="inlineStr"/>
-      <c r="G17" s="5" t="inlineStr">
+      <c r="F19" s="5" t="inlineStr"/>
+      <c r="G19" s="5" t="inlineStr">
         <is>
           <t>0905_beatenbystranger_916.mov</t>
         </is>
       </c>
-      <c r="H17" s="7" t="inlineStr">
+      <c r="H19" s="7" t="inlineStr">
         <is>
           <t>Not linked yet</t>
         </is>
       </c>
-      <c r="I17" s="5" t="inlineStr">
+      <c r="I19" s="5" t="inlineStr">
         <is>
           <t>Draft</t>
         </is>
       </c>
-      <c r="J17" s="6" t="inlineStr">
+      <c r="J19" s="6" t="inlineStr">
         <is>
           <t>my best run today. someone's already ahead of it 😭 same seed, same day, go beat them. link in bio</t>
         </is>
       </c>
-      <c r="K17" s="5" t="inlineStr">
+      <c r="K19" s="5" t="inlineStr">
         <is>
           <t>#dailychallenge #indiegame #gamingmemes #leaderboard</t>
         </is>
       </c>
-      <c r="L17" s="6" t="inlineStr">
+      <c r="L19" s="6" t="inlineStr">
         <is>
           <t>my best today. this guy's best today 💀 same run, same day, link in bio</t>
         </is>
       </c>
-      <c r="M17" s="6" t="inlineStr"/>
-      <c r="N17" s="5" t="inlineStr">
+      <c r="M19" s="6" t="inlineStr"/>
+      <c r="N19" s="5" t="inlineStr">
         <is>
           <t>Someone Already Beat My Best Run Today (ORION)</t>
         </is>
       </c>
-      <c r="O17" s="6" t="inlineStr">
+      <c r="O19" s="6" t="inlineStr">
         <is>
           <t>Same seed as every pilot. The board never sits still. Free dodging game, three attempts a day.
 Play: https://surviveorion.com
@@ -1716,70 +1854,70 @@
         </is>
       </c>
     </row>
-    <row r="18" ht="60" customHeight="1">
-      <c r="A18" s="5" t="inlineStr">
+    <row r="20" ht="60" customHeight="1">
+      <c r="A20" s="5" t="inlineStr">
         <is>
           <t>2026-09-05</t>
         </is>
       </c>
-      <c r="B18" s="5" t="inlineStr">
+      <c r="B20" s="5" t="inlineStr">
         <is>
           <t>Sat</t>
         </is>
       </c>
-      <c r="C18" s="5" t="inlineStr">
+      <c r="C20" s="5" t="inlineStr">
         <is>
           <t>TODAY'S PATROL</t>
         </is>
       </c>
-      <c r="D18" s="5" t="inlineStr">
+      <c r="D20" s="5" t="inlineStr">
         <is>
           <t>YEAR OF THE SERPENT</t>
         </is>
       </c>
-      <c r="E18" s="6" t="inlineStr">
+      <c r="E20" s="6" t="inlineStr">
         <is>
           <t>Every formation slithers today. Watch the trains.</t>
         </is>
       </c>
-      <c r="F18" s="5" t="n"/>
-      <c r="G18" s="5" t="inlineStr">
+      <c r="F20" s="5" t="n"/>
+      <c r="G20" s="5" t="inlineStr">
         <is>
           <t>0905_patrol_yearoftheserpent_916.mov</t>
         </is>
       </c>
-      <c r="H18" s="7" t="inlineStr">
+      <c r="H20" s="7" t="inlineStr">
         <is>
           <t>Not linked yet</t>
         </is>
       </c>
-      <c r="I18" s="5" t="inlineStr">
+      <c r="I20" s="5" t="inlineStr">
         <is>
           <t>Draft</t>
         </is>
       </c>
-      <c r="J18" s="6" t="inlineStr">
+      <c r="J20" s="6" t="inlineStr">
         <is>
           <t>Today every pilot flies YEAR OF THE SERPENT: Every formation slithers today. Watch the trains. Three attempts. Free, in your browser.</t>
         </is>
       </c>
-      <c r="K18" s="5" t="inlineStr">
+      <c r="K20" s="5" t="inlineStr">
         <is>
           <t>#dailychallenge #indiegame #browsergame #arcadegame</t>
         </is>
       </c>
-      <c r="L18" s="6" t="inlineStr">
+      <c r="L20" s="6" t="inlineStr">
         <is>
           <t>today every pilot flies year of the serpent: every formation slithers today. watch the trains. three attempts. free, in your browser.</t>
         </is>
       </c>
-      <c r="M18" s="6" t="n"/>
-      <c r="N18" s="5" t="inlineStr">
+      <c r="M20" s="6" t="n"/>
+      <c r="N20" s="5" t="inlineStr">
         <is>
           <t>YEAR OF THE SERPENT DAY: Today's ORION Patrol (Day 54)</t>
         </is>
       </c>
-      <c r="O18" s="6" t="inlineStr">
+      <c r="O20" s="6" t="inlineStr">
         <is>
           <t>Today's shared seed: YEAR OF THE SERPENT. No ambient drones at all. Only serpent trains, more of them, released to hunt after their sweep. Deep in the run the trains keep coming faster and stray drones start leaking in. Every pilot flies the same run. Three attempts, free in your browser.
 Play now: https://surviveorion.com
@@ -1787,74 +1925,74 @@
         </is>
       </c>
     </row>
-    <row r="19" ht="60" customHeight="1">
-      <c r="A19" s="5" t="inlineStr">
+    <row r="21" ht="60" customHeight="1">
+      <c r="A21" s="5" t="inlineStr">
         <is>
           <t>2026-09-06</t>
         </is>
       </c>
-      <c r="B19" s="5" t="inlineStr">
+      <c r="B21" s="5" t="inlineStr">
         <is>
           <t>Sun</t>
         </is>
       </c>
-      <c r="C19" s="5" t="inlineStr">
+      <c r="C21" s="5" t="inlineStr">
         <is>
           <t>TODAY'S PATROL · SUNDAY DOUBLE</t>
         </is>
       </c>
-      <c r="D19" s="5" t="inlineStr">
+      <c r="D21" s="5" t="inlineStr">
         <is>
           <t>PATROL: MAGNETIC FIELD + CLOAK</t>
         </is>
       </c>
-      <c r="E19" s="6" t="inlineStr">
+      <c r="E21" s="6" t="inlineStr">
         <is>
           <t>The pickups want to find you today. They lose the lock. You seed the dark.</t>
         </is>
       </c>
-      <c r="F19" s="5" t="inlineStr">
+      <c r="F21" s="5" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="G19" s="5" t="inlineStr">
+      <c r="G21" s="5" t="inlineStr">
         <is>
           <t>0906_patrol_magneticfieldcloak_916.mov</t>
         </is>
       </c>
-      <c r="H19" s="7" t="inlineStr">
+      <c r="H21" s="7" t="inlineStr">
         <is>
           <t>Not linked yet</t>
         </is>
       </c>
-      <c r="I19" s="5" t="inlineStr">
+      <c r="I21" s="5" t="inlineStr">
         <is>
           <t>Draft</t>
         </is>
       </c>
-      <c r="J19" s="6" t="inlineStr">
+      <c r="J21" s="6" t="inlineStr">
         <is>
           <t>Today every pilot flies MAGNETIC FIELD + CLOAK: The pickups want to find you today. They lose the lock. You seed the dark. Three attempts. Free, in your browser.</t>
         </is>
       </c>
-      <c r="K19" s="5" t="inlineStr">
+      <c r="K21" s="5" t="inlineStr">
         <is>
           <t>#dailychallenge #indiegame #browsergame #arcadegame</t>
         </is>
       </c>
-      <c r="L19" s="6" t="inlineStr">
+      <c r="L21" s="6" t="inlineStr">
         <is>
           <t>today every pilot flies magnetic field + cloak: the pickups want to find you today. they lose the lock. you seed the dark. three attempts. free, in your browser.</t>
         </is>
       </c>
-      <c r="M19" s="6" t="n"/>
-      <c r="N19" s="5" t="inlineStr">
+      <c r="M21" s="6" t="n"/>
+      <c r="N21" s="5" t="inlineStr">
         <is>
           <t>MAGNETIC FIELD + CLOAK DAY: Today's ORION Patrol (Day 55)</t>
         </is>
       </c>
-      <c r="O19" s="6" t="inlineStr">
+      <c r="O21" s="6" t="inlineStr">
         <is>
           <t>Today's shared seed: MAGNETIC FIELD + CLOAK. Pickups slowly drift toward your ship all day, on top of their normal wander. Every pickup is Cloak. Drones hover, lost. Invisible bombs drop along your path and explode when you reappear. Every pilot flies the same run. Three attempts, free in your browser.
 Play now: https://surviveorion.com
@@ -1862,70 +2000,70 @@
         </is>
       </c>
     </row>
-    <row r="20" ht="60" customHeight="1">
-      <c r="A20" s="5" t="inlineStr">
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
         <is>
           <t>2026-09-07</t>
         </is>
       </c>
-      <c r="B20" s="5" t="inlineStr">
+      <c r="B22" s="5" t="inlineStr">
         <is>
           <t>Mon</t>
         </is>
       </c>
-      <c r="C20" s="5" t="inlineStr">
+      <c r="C22" s="5" t="inlineStr">
         <is>
           <t>BUG</t>
         </is>
       </c>
-      <c r="D20" s="5" t="inlineStr">
+      <c r="D22" s="5" t="inlineStr">
         <is>
           <t>Bug of the week</t>
         </is>
       </c>
-      <c r="E20" s="6" t="inlineStr">
+      <c r="E22" s="6" t="inlineStr">
         <is>
           <t>Any real glitch, physics jank, or weird interaction. Film it as-is, matter-of-fact caption, no apology. "Who needs new features when you got old bugs."</t>
         </is>
       </c>
-      <c r="F20" s="5" t="inlineStr"/>
-      <c r="G20" s="5" t="inlineStr">
+      <c r="F22" s="5" t="inlineStr"/>
+      <c r="G22" s="5" t="inlineStr">
         <is>
           <t>0907_bugoftheweek_916.mov</t>
         </is>
       </c>
-      <c r="H20" s="7" t="inlineStr">
+      <c r="H22" s="7" t="inlineStr">
         <is>
           <t>Not linked yet</t>
         </is>
       </c>
-      <c r="I20" s="5" t="inlineStr">
+      <c r="I22" s="5" t="inlineStr">
         <is>
           <t>Draft</t>
         </is>
       </c>
-      <c r="J20" s="6" t="inlineStr">
+      <c r="J22" s="6" t="inlineStr">
         <is>
           <t>bug of the week. we see it too. free browser game, link in bio</t>
         </is>
       </c>
-      <c r="K20" s="5" t="inlineStr">
+      <c r="K22" s="5" t="inlineStr">
         <is>
           <t>#gamedev #indiegame #gamingmemes #bug</t>
         </is>
       </c>
-      <c r="L20" s="6" t="inlineStr">
+      <c r="L22" s="6" t="inlineStr">
         <is>
           <t>bug of the week 💀 nobody's perfect, free daily dodge game, link in bio</t>
         </is>
       </c>
-      <c r="M20" s="6" t="inlineStr"/>
-      <c r="N20" s="5" t="inlineStr">
+      <c r="M22" s="6" t="inlineStr"/>
+      <c r="N22" s="5" t="inlineStr">
         <is>
           <t>Bug of the Week (ORION Devlog Clip)</t>
         </is>
       </c>
-      <c r="O20" s="6" t="inlineStr">
+      <c r="O22" s="6" t="inlineStr">
         <is>
           <t>Real jank, filmed as it happened. Free daily dodging game.
 Play: https://surviveorion.com
@@ -1933,70 +2071,70 @@
         </is>
       </c>
     </row>
-    <row r="21" ht="60" customHeight="1">
-      <c r="A21" s="5" t="inlineStr">
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
         <is>
           <t>2026-09-07</t>
         </is>
       </c>
-      <c r="B21" s="5" t="inlineStr">
+      <c r="B23" s="5" t="inlineStr">
         <is>
           <t>Mon</t>
         </is>
       </c>
-      <c r="C21" s="5" t="inlineStr">
+      <c r="C23" s="5" t="inlineStr">
         <is>
           <t>TODAY'S PATROL</t>
         </is>
       </c>
-      <c r="D21" s="5" t="inlineStr">
+      <c r="D23" s="5" t="inlineStr">
         <is>
           <t>RAM RAID</t>
         </is>
       </c>
-      <c r="E21" s="6" t="inlineStr">
+      <c r="E23" s="6" t="inlineStr">
         <is>
           <t>The shell is short. Spend it, then dodge naked.</t>
         </is>
       </c>
-      <c r="F21" s="5" t="n"/>
-      <c r="G21" s="5" t="inlineStr">
+      <c r="F23" s="5" t="n"/>
+      <c r="G23" s="5" t="inlineStr">
         <is>
           <t>0907_patrol_ramraid_916.mov</t>
         </is>
       </c>
-      <c r="H21" s="7" t="inlineStr">
+      <c r="H23" s="7" t="inlineStr">
         <is>
           <t>Not linked yet</t>
         </is>
       </c>
-      <c r="I21" s="5" t="inlineStr">
+      <c r="I23" s="5" t="inlineStr">
         <is>
           <t>Draft</t>
         </is>
       </c>
-      <c r="J21" s="6" t="inlineStr">
+      <c r="J23" s="6" t="inlineStr">
         <is>
           <t>Today every pilot flies RAM RAID: The shell is short. Spend it, then dodge naked. Three attempts. Free, in your browser.</t>
         </is>
       </c>
-      <c r="K21" s="5" t="inlineStr">
+      <c r="K23" s="5" t="inlineStr">
         <is>
           <t>#dailychallenge #indiegame #browsergame #arcadegame</t>
         </is>
       </c>
-      <c r="L21" s="6" t="inlineStr">
+      <c r="L23" s="6" t="inlineStr">
         <is>
           <t>today every pilot flies ram raid: the shell is short. spend it, then dodge naked. three attempts. free, in your browser.</t>
         </is>
       </c>
-      <c r="M21" s="6" t="n"/>
-      <c r="N21" s="5" t="inlineStr">
+      <c r="M23" s="6" t="n"/>
+      <c r="N23" s="5" t="inlineStr">
         <is>
           <t>RAM RAID DAY: Today's ORION Patrol (Day 56)</t>
         </is>
       </c>
-      <c r="O21" s="6" t="inlineStr">
+      <c r="O23" s="6" t="inlineStr">
         <is>
           <t>Today's shared seed: RAM RAID. Starshell is the only drop, and it is scarce. The shell lasts about two seconds. You are invincible while it is up. Every pilot flies the same run. Three attempts, free in your browser.
 Play now: https://surviveorion.com
@@ -2004,70 +2142,70 @@
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="5" t="inlineStr">
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
         <is>
           <t>2026-09-08</t>
         </is>
       </c>
-      <c r="B22" s="5" t="inlineStr">
+      <c r="B24" s="5" t="inlineStr">
         <is>
           <t>Tue</t>
         </is>
       </c>
-      <c r="C22" s="5" t="inlineStr">
+      <c r="C24" s="5" t="inlineStr">
         <is>
           <t>TODAY'S PATROL</t>
         </is>
       </c>
-      <c r="D22" s="5" t="inlineStr">
+      <c r="D24" s="5" t="inlineStr">
         <is>
           <t>SINGULARITY</t>
         </is>
       </c>
-      <c r="E22" s="6" t="inlineStr">
+      <c r="E24" s="6" t="inlineStr">
         <is>
           <t>The banned singularity is back for one day. Use it well.</t>
         </is>
       </c>
-      <c r="F22" s="5" t="n"/>
-      <c r="G22" s="5" t="inlineStr">
+      <c r="F24" s="5" t="n"/>
+      <c r="G24" s="5" t="inlineStr">
         <is>
           <t>0908_patrol_singularity_916.mov</t>
         </is>
       </c>
-      <c r="H22" s="7" t="inlineStr">
+      <c r="H24" s="7" t="inlineStr">
         <is>
           <t>Not linked yet</t>
         </is>
       </c>
-      <c r="I22" s="5" t="inlineStr">
+      <c r="I24" s="5" t="inlineStr">
         <is>
           <t>Draft</t>
         </is>
       </c>
-      <c r="J22" s="6" t="inlineStr">
+      <c r="J24" s="6" t="inlineStr">
         <is>
           <t>Today every pilot flies SINGULARITY: The banned singularity is back for one day. Use it well. Three attempts. Free, in your browser.</t>
         </is>
       </c>
-      <c r="K22" s="5" t="inlineStr">
+      <c r="K24" s="5" t="inlineStr">
         <is>
           <t>#dailychallenge #indiegame #browsergame #arcadegame</t>
         </is>
       </c>
-      <c r="L22" s="6" t="inlineStr">
+      <c r="L24" s="6" t="inlineStr">
         <is>
           <t>today every pilot flies singularity: the banned singularity is back for one day. use it well. three attempts. free, in your browser.</t>
         </is>
       </c>
-      <c r="M22" s="6" t="n"/>
-      <c r="N22" s="5" t="inlineStr">
+      <c r="M24" s="6" t="n"/>
+      <c r="N24" s="5" t="inlineStr">
         <is>
           <t>SINGULARITY DAY: Today's ORION Patrol (Day 57)</t>
         </is>
       </c>
-      <c r="O22" s="6" t="inlineStr">
+      <c r="O24" s="6" t="inlineStr">
         <is>
           <t>Today's shared seed: SINGULARITY. Vortex (normally benched) drops often today. Every pilot flies the same run. Three attempts, free in your browser.
 Play now: https://surviveorion.com
@@ -2075,68 +2213,68 @@
         </is>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
+    <row r="25">
+      <c r="A25" t="inlineStr">
         <is>
           <t>2026-09-26</t>
         </is>
       </c>
-      <c r="B23" t="inlineStr">
+      <c r="B25" t="inlineStr">
         <is>
           <t>Sat</t>
         </is>
       </c>
-      <c r="C23" t="inlineStr">
+      <c r="C25" t="inlineStr">
         <is>
           <t>TODAY'S PATROL</t>
         </is>
       </c>
-      <c r="D23" t="inlineStr">
+      <c r="D25" t="inlineStr">
         <is>
           <t>GREAT WALL</t>
         </is>
       </c>
-      <c r="E23" t="inlineStr">
+      <c r="E25" t="inlineStr">
         <is>
           <t>nothing but walls today.</t>
         </is>
       </c>
-      <c r="G23" t="inlineStr">
+      <c r="G25" t="inlineStr">
         <is>
           <t>0827_greatwall_916.mov</t>
         </is>
       </c>
-      <c r="H23" t="inlineStr">
+      <c r="H25" t="inlineStr">
         <is>
           <t>Linked</t>
         </is>
       </c>
-      <c r="I23" t="inlineStr">
+      <c r="I25" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
       </c>
-      <c r="J23" t="inlineStr">
+      <c r="J25" t="inlineStr">
         <is>
           <t>Today every pilot flies GREAT WALL: nothing but walls today. Three attempts. Free, in your browser.</t>
         </is>
       </c>
-      <c r="K23" t="inlineStr">
+      <c r="K25" t="inlineStr">
         <is>
           <t>#dailychallenge #indiegame #browsergame #arcadegame</t>
         </is>
       </c>
-      <c r="L23" t="inlineStr">
+      <c r="L25" t="inlineStr">
         <is>
           <t>today every pilot flies great wall: nothing but walls today. three attempts. free, in your browser.</t>
         </is>
       </c>
-      <c r="N23" t="inlineStr">
+      <c r="N25" t="inlineStr">
         <is>
           <t>GREAT WALL DAY: Today's ORION Patrol (Day 75)</t>
         </is>
       </c>
-      <c r="O23" t="inlineStr">
+      <c r="O25" t="inlineStr">
         <is>
           <t>Today's shared seed: GREAT WALL. No ambient drones at all. Only walls, mega walls, and pincers, faster than usual, released to hunt after their sweep. Every pilot flies the same run. Three attempts, free in your browser.
 Play now: https://surviveorion.com

</xml_diff>

<commit_message>
Mark Ditch the Can and Dead Fart as scheduled. [skip render]
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/ORION_Publishing_Calendar.xlsx
+++ b/ORION_Publishing_Calendar.xlsx
@@ -1327,7 +1327,7 @@
       </c>
       <c r="I12" s="5" t="inlineStr">
         <is>
-          <t>Approved</t>
+          <t>Scheduled</t>
         </is>
       </c>
       <c r="J12" s="6" t="inlineStr">
@@ -1467,7 +1467,7 @@
       </c>
       <c r="I14" s="5" t="inlineStr">
         <is>
-          <t>Approved</t>
+          <t>Scheduled</t>
         </is>
       </c>
       <c r="J14" s="6" t="inlineStr">

</xml_diff>

<commit_message>
Rewrite Ditch the Can and Dead Fart captions. [skip render]
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/ORION_Publishing_Calendar.xlsx
+++ b/ORION_Publishing_Calendar.xlsx
@@ -1311,7 +1311,7 @@
       </c>
       <c r="E12" s="6" t="inlineStr">
         <is>
-          <t>Bored? Ditch the can</t>
+          <t>The can is not content.</t>
         </is>
       </c>
       <c r="F12" s="5" t="n"/>
@@ -1332,7 +1332,7 @@
       </c>
       <c r="J12" s="6" t="inlineStr">
         <is>
-          <t>Bored? Ditch the can. Play ORION instead 🛰️ Daily dodge, three attempts, free. Link in bio.</t>
+          <t>Caught myself reading a bathroom can like it was a novel 🚽📖 There's a better daily. Three attempts. Free. 🛰️⚡ Link in bio.</t>
         </is>
       </c>
       <c r="K12" s="5" t="inlineStr">
@@ -1342,18 +1342,18 @@
       </c>
       <c r="L12" s="6" t="inlineStr">
         <is>
-          <t>bored? ditch the can. play orion instead 💀 free daily dodge game, 3 attempts, link in bio</t>
+          <t>caught myself studying a bathroom can like it was homework so i found a daily dodge game instead 🚽💀🛰️ 3 attempts, free, link in bio</t>
         </is>
       </c>
       <c r="M12" s="6" t="n"/>
       <c r="N12" s="5" t="inlineStr">
         <is>
-          <t>Bored? Ditch the Can. Play ORION Instead</t>
+          <t>There's a Better Daily Than the Bathroom Can</t>
         </is>
       </c>
       <c r="O12" s="6" t="inlineStr">
         <is>
-          <t>Reading the can again? Daily dodge game. Three attempts, same run as every other pilot. It's free.
+          <t>The can is not content. Same swarm as every other pilot, three attempts, it's free.
 Play: https://surviveorion.com
 #gamingmemes #indiegame #Shorts</t>
         </is>
@@ -1451,7 +1451,7 @@
       </c>
       <c r="E14" s="6" t="inlineStr">
         <is>
-          <t>he died. the game farted.</t>
+          <t>You don't say Ray.</t>
         </is>
       </c>
       <c r="F14" s="5" t="n"/>
@@ -1472,7 +1472,10 @@
       </c>
       <c r="J14" s="6" t="inlineStr">
         <is>
-          <t>he died. the game farted. 💀 Free daily dodge game, link in bio.</t>
+          <t>"There is no trap so deadly as the trap you set for yourself."
+Raymond Chandler.
+You don't say Ray 💀💨
+Free daily dodge. Link in bio.</t>
         </is>
       </c>
       <c r="K14" s="5" t="inlineStr">
@@ -1482,18 +1485,21 @@
       </c>
       <c r="L14" s="6" t="inlineStr">
         <is>
-          <t>he died. the game farted. 💀 free daily dodge game, 3 attempts, link in bio</t>
+          <t>"there is no trap so deadly as the trap you set for yourself" raymond chandler
+you don't say ray 💀💨
+free daily dodge game, link in bio</t>
         </is>
       </c>
       <c r="M14" s="6" t="n"/>
       <c r="N14" s="5" t="inlineStr">
         <is>
-          <t>He Died. The Game Farted. (ORION)</t>
+          <t>You Don't Say Ray (ORION)</t>
         </is>
       </c>
       <c r="O14" s="6" t="inlineStr">
         <is>
-          <t>The daily patrol remains undefeated. The sound design had opinions.
+          <t>"There is no trap so deadly as the trap you set for yourself." Raymond Chandler.
+You don't say Ray.
 Play: https://surviveorion.com
 #Shorts</t>
         </is>

</xml_diff>

<commit_message>
Make Ditch the Can second person. [skip render]
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/ORION_Publishing_Calendar.xlsx
+++ b/ORION_Publishing_Calendar.xlsx
@@ -1332,7 +1332,7 @@
       </c>
       <c r="J12" s="6" t="inlineStr">
         <is>
-          <t>Caught myself reading a bathroom can like it was a novel 🚽📖 There's a better daily. Three attempts. Free. 🛰️⚡ Link in bio.</t>
+          <t>Caught yourself reading a bathroom can like it was a novel? 🚽📖 There's a better daily. Three attempts. Free. 🛰️⚡ Link in bio.</t>
         </is>
       </c>
       <c r="K12" s="5" t="inlineStr">
@@ -1342,7 +1342,7 @@
       </c>
       <c r="L12" s="6" t="inlineStr">
         <is>
-          <t>caught myself studying a bathroom can like it was homework so i found a daily dodge game instead 🚽💀🛰️ 3 attempts, free, link in bio</t>
+          <t>caught yourself reading a bathroom can like it was a novel? 🚽📖 there's a better daily. 3 attempts, free, link in bio</t>
         </is>
       </c>
       <c r="M12" s="6" t="n"/>

</xml_diff>